<commit_message>
Historicos: backfill de los 4 LECER nuevos desde series de 1816
Agrega columnas TZXY7, X30N6, X31L6, X30S6 con precioDirty histórico traído de
/v1/mercado/series (moneda ars), alineado a las 40 fechas del histórico.
X30N6 tiene dato al 2025-12-30 (94) => su YTD se calcula (+28.04%). TZXY7 no
cotizó a fin de 2025 y X31L6/X30S6 se emitieron en 2026 => YTD "—" (correcto).

historicos.xlsx no tiene fórmulas, así que se editó con openpyxl sin riesgo
(a diferencia de Instrumentos.xlsx). De acá en adelante el job diario los
actualiza solo, porque ya están en Instrumentos.xlsx.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/historicos.xlsx
+++ b/historicos.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="760" windowWidth="29400" windowHeight="16980" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Historicos" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Historicos" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CA41"/>
+  <dimension ref="A1:CE41"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="15"/>
   <cols>
     <col width="10.6640625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -817,6 +817,26 @@
           <t>AO29D</t>
         </is>
       </c>
+      <c r="CB1" t="inlineStr">
+        <is>
+          <t>TZXY7</t>
+        </is>
+      </c>
+      <c r="CC1" t="inlineStr">
+        <is>
+          <t>X30N6</t>
+        </is>
+      </c>
+      <c r="CD1" t="inlineStr">
+        <is>
+          <t>X31L6</t>
+        </is>
+      </c>
+      <c r="CE1" t="inlineStr">
+        <is>
+          <t>X30S6</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
@@ -1038,6 +1058,9 @@
       <c r="BU2" t="n">
         <v>79.59999999999999</v>
       </c>
+      <c r="CC2" t="n">
+        <v>94</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1222,6 +1245,18 @@
       <c r="BH3" t="n">
         <v>158.7</v>
       </c>
+      <c r="CB3" t="n">
+        <v>113.7</v>
+      </c>
+      <c r="CC3" t="n">
+        <v>117.15</v>
+      </c>
+      <c r="CD3" t="n">
+        <v>113.5</v>
+      </c>
+      <c r="CE3" t="n">
+        <v>108.801</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1406,6 +1441,18 @@
       <c r="BH4" t="n">
         <v>158.5</v>
       </c>
+      <c r="CB4" t="n">
+        <v>113.7</v>
+      </c>
+      <c r="CC4" t="n">
+        <v>117.25</v>
+      </c>
+      <c r="CD4" t="n">
+        <v>113.5</v>
+      </c>
+      <c r="CE4" t="n">
+        <v>108.95</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1587,6 +1634,18 @@
       <c r="BH5" t="n">
         <v>158.6</v>
       </c>
+      <c r="CB5" t="n">
+        <v>114</v>
+      </c>
+      <c r="CC5" t="n">
+        <v>117.295</v>
+      </c>
+      <c r="CD5" t="n">
+        <v>113.8</v>
+      </c>
+      <c r="CE5" t="n">
+        <v>109</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1792,6 +1851,18 @@
       <c r="BP6" t="n">
         <v>109</v>
       </c>
+      <c r="CB6" t="n">
+        <v>114.35</v>
+      </c>
+      <c r="CC6" t="n">
+        <v>117.7</v>
+      </c>
+      <c r="CD6" t="n">
+        <v>113.9</v>
+      </c>
+      <c r="CE6" t="n">
+        <v>109.3</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1997,6 +2068,18 @@
       <c r="BP7" t="n">
         <v>105.3</v>
       </c>
+      <c r="CB7" t="n">
+        <v>114.6</v>
+      </c>
+      <c r="CC7" t="n">
+        <v>117.8</v>
+      </c>
+      <c r="CD7" t="n">
+        <v>114.25</v>
+      </c>
+      <c r="CE7" t="n">
+        <v>109.37</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -2202,6 +2285,18 @@
       <c r="BP8" t="n">
         <v>102.8</v>
       </c>
+      <c r="CB8" t="n">
+        <v>115.1</v>
+      </c>
+      <c r="CC8" t="n">
+        <v>117.815</v>
+      </c>
+      <c r="CD8" t="n">
+        <v>114.3</v>
+      </c>
+      <c r="CE8" t="n">
+        <v>109.32</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -2407,6 +2502,18 @@
       <c r="BP9" t="n">
         <v>105.1</v>
       </c>
+      <c r="CB9" t="n">
+        <v>114.95</v>
+      </c>
+      <c r="CC9" t="n">
+        <v>117.7</v>
+      </c>
+      <c r="CD9" t="n">
+        <v>114.2</v>
+      </c>
+      <c r="CE9" t="n">
+        <v>109.3</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2612,6 +2719,18 @@
       <c r="BP10" t="n">
         <v>105.65</v>
       </c>
+      <c r="CB10" t="n">
+        <v>115.1</v>
+      </c>
+      <c r="CC10" t="n">
+        <v>117.76</v>
+      </c>
+      <c r="CD10" t="n">
+        <v>114.225</v>
+      </c>
+      <c r="CE10" t="n">
+        <v>109.45</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -2814,6 +2933,18 @@
       <c r="BP11" t="n">
         <v>105.55</v>
       </c>
+      <c r="CB11" t="n">
+        <v>115.3</v>
+      </c>
+      <c r="CC11" t="n">
+        <v>118.2</v>
+      </c>
+      <c r="CD11" t="n">
+        <v>114.452</v>
+      </c>
+      <c r="CE11" t="n">
+        <v>109.65</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -3016,6 +3147,18 @@
       <c r="BP12" t="n">
         <v>105.9</v>
       </c>
+      <c r="CB12" t="n">
+        <v>115.75</v>
+      </c>
+      <c r="CC12" t="n">
+        <v>118.34</v>
+      </c>
+      <c r="CD12" t="n">
+        <v>114.5</v>
+      </c>
+      <c r="CE12" t="n">
+        <v>109.71</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -3218,6 +3361,18 @@
       <c r="BP13" t="n">
         <v>105.8</v>
       </c>
+      <c r="CB13" t="n">
+        <v>116</v>
+      </c>
+      <c r="CC13" t="n">
+        <v>118.75</v>
+      </c>
+      <c r="CD13" t="n">
+        <v>114.65</v>
+      </c>
+      <c r="CE13" t="n">
+        <v>111</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -3420,6 +3575,18 @@
       <c r="BP14" t="n">
         <v>105.45</v>
       </c>
+      <c r="CB14" t="n">
+        <v>116.2</v>
+      </c>
+      <c r="CC14" t="n">
+        <v>118.775</v>
+      </c>
+      <c r="CD14" t="n">
+        <v>114.727</v>
+      </c>
+      <c r="CE14" t="n">
+        <v>110.25</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -3619,6 +3786,18 @@
       <c r="BP15" t="n">
         <v>105.25</v>
       </c>
+      <c r="CB15" t="n">
+        <v>116.3</v>
+      </c>
+      <c r="CC15" t="n">
+        <v>118.8</v>
+      </c>
+      <c r="CD15" t="n">
+        <v>114.8</v>
+      </c>
+      <c r="CE15" t="n">
+        <v>110.25</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -3833,6 +4012,18 @@
       <c r="BU16" t="n">
         <v>79.59999999999999</v>
       </c>
+      <c r="CB16" t="n">
+        <v>116.9</v>
+      </c>
+      <c r="CC16" t="n">
+        <v>118.65</v>
+      </c>
+      <c r="CD16" t="n">
+        <v>114.81</v>
+      </c>
+      <c r="CE16" t="n">
+        <v>110.25</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -4261,6 +4452,18 @@
       <c r="BU18" t="n">
         <v>79.7</v>
       </c>
+      <c r="CB18" t="n">
+        <v>116.8</v>
+      </c>
+      <c r="CC18" t="n">
+        <v>118.45</v>
+      </c>
+      <c r="CD18" t="n">
+        <v>114.8</v>
+      </c>
+      <c r="CE18" t="n">
+        <v>110.1</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -4475,6 +4678,18 @@
       <c r="BU19" t="n">
         <v>79.09999999999999</v>
       </c>
+      <c r="CB19" t="n">
+        <v>116.8</v>
+      </c>
+      <c r="CC19" t="n">
+        <v>118.2</v>
+      </c>
+      <c r="CD19" t="n">
+        <v>114.85</v>
+      </c>
+      <c r="CE19" t="n">
+        <v>110.1</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -4689,6 +4904,18 @@
       <c r="BU20" t="n">
         <v>79.05</v>
       </c>
+      <c r="CB20" t="n">
+        <v>116</v>
+      </c>
+      <c r="CC20" t="n">
+        <v>118.35</v>
+      </c>
+      <c r="CD20" t="n">
+        <v>114.88</v>
+      </c>
+      <c r="CE20" t="n">
+        <v>110.25</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -4903,6 +5130,18 @@
       <c r="BU21" t="n">
         <v>79.08</v>
       </c>
+      <c r="CB21" t="n">
+        <v>116</v>
+      </c>
+      <c r="CC21" t="n">
+        <v>118.301</v>
+      </c>
+      <c r="CD21" t="n">
+        <v>115.21</v>
+      </c>
+      <c r="CE21" t="n">
+        <v>110.35</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -5117,6 +5356,18 @@
       <c r="BU22" t="n">
         <v>79.14</v>
       </c>
+      <c r="CB22" t="n">
+        <v>116.5</v>
+      </c>
+      <c r="CC22" t="n">
+        <v>118.5</v>
+      </c>
+      <c r="CD22" t="n">
+        <v>115.25</v>
+      </c>
+      <c r="CE22" t="n">
+        <v>110.499</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -5331,6 +5582,18 @@
       <c r="BU23" t="n">
         <v>79.09</v>
       </c>
+      <c r="CB23" t="n">
+        <v>116</v>
+      </c>
+      <c r="CC23" t="n">
+        <v>118.4</v>
+      </c>
+      <c r="CD23" t="n">
+        <v>115.3</v>
+      </c>
+      <c r="CE23" t="n">
+        <v>110.4</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -5545,6 +5808,18 @@
       <c r="BU24" t="n">
         <v>79.63</v>
       </c>
+      <c r="CB24" t="n">
+        <v>115.75</v>
+      </c>
+      <c r="CC24" t="n">
+        <v>118.38</v>
+      </c>
+      <c r="CD24" t="n">
+        <v>115.3</v>
+      </c>
+      <c r="CE24" t="n">
+        <v>110.45</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -5759,6 +6034,18 @@
       <c r="BU25" t="n">
         <v>79.2</v>
       </c>
+      <c r="CB25" t="n">
+        <v>115.4</v>
+      </c>
+      <c r="CC25" t="n">
+        <v>118.25</v>
+      </c>
+      <c r="CD25" t="n">
+        <v>115.3</v>
+      </c>
+      <c r="CE25" t="n">
+        <v>110.45</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -5973,6 +6260,18 @@
       <c r="BU26" t="n">
         <v>79.40000000000001</v>
       </c>
+      <c r="CB26" t="n">
+        <v>115.8</v>
+      </c>
+      <c r="CC26" t="n">
+        <v>118.55</v>
+      </c>
+      <c r="CD26" t="n">
+        <v>115.52</v>
+      </c>
+      <c r="CE26" t="n">
+        <v>110.55</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -6175,6 +6474,18 @@
       <c r="BU27" t="n">
         <v>79.8</v>
       </c>
+      <c r="CB27" t="n">
+        <v>116.45</v>
+      </c>
+      <c r="CC27" t="n">
+        <v>118.77</v>
+      </c>
+      <c r="CD27" t="n">
+        <v>115.65</v>
+      </c>
+      <c r="CE27" t="n">
+        <v>111</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -6389,6 +6700,18 @@
       <c r="BY28" t="n">
         <v>101.7</v>
       </c>
+      <c r="CB28" t="n">
+        <v>116.3</v>
+      </c>
+      <c r="CC28" t="n">
+        <v>118.9</v>
+      </c>
+      <c r="CD28" t="n">
+        <v>115.852</v>
+      </c>
+      <c r="CE28" t="n">
+        <v>110.93</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -6603,6 +6926,18 @@
       <c r="BY29" t="n">
         <v>101.6</v>
       </c>
+      <c r="CB29" t="n">
+        <v>116.3</v>
+      </c>
+      <c r="CC29" t="n">
+        <v>118.9</v>
+      </c>
+      <c r="CD29" t="n">
+        <v>116.04</v>
+      </c>
+      <c r="CE29" t="n">
+        <v>111.05</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -6817,6 +7152,18 @@
       <c r="BY30" t="n">
         <v>101.7</v>
       </c>
+      <c r="CB30" t="n">
+        <v>116.3</v>
+      </c>
+      <c r="CC30" t="n">
+        <v>119.07</v>
+      </c>
+      <c r="CD30" t="n">
+        <v>116.031</v>
+      </c>
+      <c r="CE30" t="n">
+        <v>111</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -7031,6 +7378,18 @@
       <c r="BY31" t="n">
         <v>102.3</v>
       </c>
+      <c r="CB31" t="n">
+        <v>116.5</v>
+      </c>
+      <c r="CC31" t="n">
+        <v>119.412</v>
+      </c>
+      <c r="CD31" t="n">
+        <v>116.25</v>
+      </c>
+      <c r="CE31" t="n">
+        <v>111.15</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -7245,6 +7604,18 @@
       <c r="BY32" t="n">
         <v>102.5</v>
       </c>
+      <c r="CB32" t="n">
+        <v>116.15</v>
+      </c>
+      <c r="CC32" t="n">
+        <v>119.675</v>
+      </c>
+      <c r="CD32" t="n">
+        <v>116.35</v>
+      </c>
+      <c r="CE32" t="n">
+        <v>111.4</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -7459,6 +7830,18 @@
       <c r="BY33" t="n">
         <v>102.8</v>
       </c>
+      <c r="CB33" t="n">
+        <v>116.9</v>
+      </c>
+      <c r="CC33" t="n">
+        <v>119.6</v>
+      </c>
+      <c r="CD33" t="n">
+        <v>116.39</v>
+      </c>
+      <c r="CE33" t="n">
+        <v>111.4</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -7673,6 +8056,18 @@
       <c r="BY34" t="n">
         <v>102.9</v>
       </c>
+      <c r="CB34" t="n">
+        <v>116.9</v>
+      </c>
+      <c r="CC34" t="n">
+        <v>119.95</v>
+      </c>
+      <c r="CD34" t="n">
+        <v>116.71</v>
+      </c>
+      <c r="CE34" t="n">
+        <v>111.52</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -8101,6 +8496,18 @@
       <c r="BY36" t="n">
         <v>104</v>
       </c>
+      <c r="CB36" t="n">
+        <v>117.9</v>
+      </c>
+      <c r="CC36" t="n">
+        <v>120.112</v>
+      </c>
+      <c r="CD36" t="n">
+        <v>116.9</v>
+      </c>
+      <c r="CE36" t="n">
+        <v>111.989</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -8315,6 +8722,18 @@
       <c r="BY37" t="n">
         <v>102.9</v>
       </c>
+      <c r="CB37" t="n">
+        <v>116.8</v>
+      </c>
+      <c r="CC37" t="n">
+        <v>119.9</v>
+      </c>
+      <c r="CD37" t="n">
+        <v>116.75</v>
+      </c>
+      <c r="CE37" t="n">
+        <v>111.749</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -8529,6 +8948,18 @@
       <c r="BY38" t="n">
         <v>103</v>
       </c>
+      <c r="CB38" t="n">
+        <v>116.8</v>
+      </c>
+      <c r="CC38" t="n">
+        <v>119.95</v>
+      </c>
+      <c r="CD38" t="n">
+        <v>116.8</v>
+      </c>
+      <c r="CE38" t="n">
+        <v>111.78</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -8743,6 +9174,18 @@
       <c r="BY39" t="n">
         <v>103.75</v>
       </c>
+      <c r="CB39" t="n">
+        <v>117.2</v>
+      </c>
+      <c r="CC39" t="n">
+        <v>119.871</v>
+      </c>
+      <c r="CD39" t="n">
+        <v>117</v>
+      </c>
+      <c r="CE39" t="n">
+        <v>111.95</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -8954,6 +9397,18 @@
       <c r="BY40" t="n">
         <v>103.3</v>
       </c>
+      <c r="CB40" t="n">
+        <v>116.8</v>
+      </c>
+      <c r="CC40" t="n">
+        <v>120.14</v>
+      </c>
+      <c r="CD40" t="n">
+        <v>117.01</v>
+      </c>
+      <c r="CE40" t="n">
+        <v>112.049</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -9170,6 +9625,18 @@
       </c>
       <c r="CA41" t="n">
         <v>94.64000000000001</v>
+      </c>
+      <c r="CB41" t="n">
+        <v>116.5</v>
+      </c>
+      <c r="CC41" t="n">
+        <v>120.36</v>
+      </c>
+      <c r="CD41" t="n">
+        <v>117.2</v>
+      </c>
+      <c r="CE41" t="n">
+        <v>112.19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Revertir la fila 2026-07-20 (corrida manual antes de la apertura)
La corrida manual del workflow (~09:42 ART) se ejecutó antes de que abriera el
mercado, así que 1816 no tenía datos para hoy ("1816: 0 precios obtenidos de 73")
y el script cayó al fallback de Eco, escribiendo una fila 2026-07-20 con los
cierres del viernes.

El problema: actualizar_historicos.py sale sin hacer nada si ya existe la fila
del día ("Ya existe fila para {fecha}, saliendo"), así que la corrida real del
cron de hoy a las 17:05 se saltearía el día y se perdería el cierre del lunes.
Se elimina la fila para que el cron la escriba con datos reales de 1816.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/historicos.xlsx
+++ b/historicos.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="760" windowWidth="29400" windowHeight="16980" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Historicos" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Historicos" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CE42"/>
+  <dimension ref="A1:CE41"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="15"/>
   <cols>
     <col width="10.6640625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -9639,232 +9639,6 @@
         <v>112.19</v>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>2026-07-20</t>
-        </is>
-      </c>
-      <c r="F42" t="n">
-        <v>117.1</v>
-      </c>
-      <c r="G42" t="n">
-        <v>106.48</v>
-      </c>
-      <c r="H42" t="n">
-        <v>124</v>
-      </c>
-      <c r="I42" t="n">
-        <v>112.599</v>
-      </c>
-      <c r="J42" t="n">
-        <v>127.25</v>
-      </c>
-      <c r="K42" t="n">
-        <v>119.64</v>
-      </c>
-      <c r="L42" t="n">
-        <v>144.34</v>
-      </c>
-      <c r="M42" t="n">
-        <v>131.72</v>
-      </c>
-      <c r="N42" t="n">
-        <v>124.45</v>
-      </c>
-      <c r="O42" t="n">
-        <v>126.19</v>
-      </c>
-      <c r="P42" t="n">
-        <v>102</v>
-      </c>
-      <c r="Q42" t="n">
-        <v>113.2</v>
-      </c>
-      <c r="S42" t="n">
-        <v>166.3</v>
-      </c>
-      <c r="T42" t="n">
-        <v>292.5</v>
-      </c>
-      <c r="U42" t="n">
-        <v>215.7</v>
-      </c>
-      <c r="V42" t="n">
-        <v>119.45</v>
-      </c>
-      <c r="W42" t="n">
-        <v>384.5</v>
-      </c>
-      <c r="X42" t="n">
-        <v>103.55</v>
-      </c>
-      <c r="Y42" t="n">
-        <v>268.7</v>
-      </c>
-      <c r="Z42" t="n">
-        <v>97.34999999999999</v>
-      </c>
-      <c r="AA42" t="n">
-        <v>344.05</v>
-      </c>
-      <c r="AB42" t="n">
-        <v>93.45999999999999</v>
-      </c>
-      <c r="AC42" t="n">
-        <v>89.89</v>
-      </c>
-      <c r="AD42" t="n">
-        <v>126.53</v>
-      </c>
-      <c r="AE42" t="n">
-        <v>117.2</v>
-      </c>
-      <c r="AF42" t="n">
-        <v>110.5</v>
-      </c>
-      <c r="AG42" t="n">
-        <v>107.45</v>
-      </c>
-      <c r="AH42" t="n">
-        <v>104.1</v>
-      </c>
-      <c r="AJ42" t="n">
-        <v>146550</v>
-      </c>
-      <c r="AK42" t="n">
-        <v>144700</v>
-      </c>
-      <c r="AL42" t="n">
-        <v>126840</v>
-      </c>
-      <c r="AM42" t="n">
-        <v>102.7</v>
-      </c>
-      <c r="AN42" t="n">
-        <v>97.89</v>
-      </c>
-      <c r="AO42" t="n">
-        <v>55.37</v>
-      </c>
-      <c r="AP42" t="n">
-        <v>97.15000000000001</v>
-      </c>
-      <c r="AQ42" t="n">
-        <v>56.47</v>
-      </c>
-      <c r="AR42" t="n">
-        <v>80.81999999999999</v>
-      </c>
-      <c r="AS42" t="n">
-        <v>83.64</v>
-      </c>
-      <c r="AT42" t="n">
-        <v>76.91</v>
-      </c>
-      <c r="AU42" t="n">
-        <v>55.95</v>
-      </c>
-      <c r="AV42" t="n">
-        <v>57.99</v>
-      </c>
-      <c r="AW42" t="n">
-        <v>83.56999999999999</v>
-      </c>
-      <c r="AX42" t="n">
-        <v>86.89</v>
-      </c>
-      <c r="AY42" t="n">
-        <v>77.98</v>
-      </c>
-      <c r="AZ42" t="n">
-        <v>72.06999999999999</v>
-      </c>
-      <c r="BA42" t="n">
-        <v>102.65</v>
-      </c>
-      <c r="BB42" t="n">
-        <v>102.6</v>
-      </c>
-      <c r="BC42" t="n">
-        <v>93.09</v>
-      </c>
-      <c r="BD42" t="n">
-        <v>92.8</v>
-      </c>
-      <c r="BE42" t="n">
-        <v>96.65000000000001</v>
-      </c>
-      <c r="BF42" t="n">
-        <v>91.09999999999999</v>
-      </c>
-      <c r="BH42" t="n">
-        <v>163.8</v>
-      </c>
-      <c r="BI42" t="n">
-        <v>103.59</v>
-      </c>
-      <c r="BJ42" t="n">
-        <v>147290</v>
-      </c>
-      <c r="BK42" t="n">
-        <v>145540</v>
-      </c>
-      <c r="BM42" t="n">
-        <v>104</v>
-      </c>
-      <c r="BN42" t="n">
-        <v>105</v>
-      </c>
-      <c r="BO42" t="n">
-        <v>112.7</v>
-      </c>
-      <c r="BP42" t="n">
-        <v>108</v>
-      </c>
-      <c r="BQ42" t="n">
-        <v>146750</v>
-      </c>
-      <c r="BR42" t="n">
-        <v>120500</v>
-      </c>
-      <c r="BS42" t="n">
-        <v>92.05</v>
-      </c>
-      <c r="BT42" t="n">
-        <v>85.09</v>
-      </c>
-      <c r="BU42" t="n">
-        <v>82.3</v>
-      </c>
-      <c r="BV42" t="n">
-        <v>102.06</v>
-      </c>
-      <c r="BW42" t="n">
-        <v>93.59999999999999</v>
-      </c>
-      <c r="BX42" t="n">
-        <v>84.09999999999999</v>
-      </c>
-      <c r="BY42" t="n">
-        <v>103.1</v>
-      </c>
-      <c r="BZ42" t="n">
-        <v>146600</v>
-      </c>
-      <c r="CA42" t="n">
-        <v>94.64</v>
-      </c>
-      <c r="CB42" t="n">
-        <v>116.5</v>
-      </c>
-      <c r="CC42" t="n">
-        <v>120.36</v>
-      </c>
-      <c r="CE42" t="n">
-        <v>112.19</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Completar ruedas incompletas 2026-08-14
</commit_message>
<xml_diff>
--- a/historicos.xlsx
+++ b/historicos.xlsx
@@ -24985,6 +24985,18 @@
       <c r="BK53" t="n">
         <v>146500</v>
       </c>
+      <c r="BM53" t="n">
+        <v>101.8</v>
+      </c>
+      <c r="BN53" t="n">
+        <v>107.7</v>
+      </c>
+      <c r="BO53" t="n">
+        <v>113.6</v>
+      </c>
+      <c r="BP53" t="n">
+        <v>108.1</v>
+      </c>
       <c r="BQ53" t="n">
         <v>148450</v>
       </c>
@@ -25033,6 +25045,252 @@
       <c r="CG53" t="n">
         <v>102.4</v>
       </c>
+      <c r="CH53" t="n">
+        <v>47.8</v>
+      </c>
+      <c r="CI53" t="n">
+        <v>63.9</v>
+      </c>
+      <c r="CJ53" t="n">
+        <v>112.1</v>
+      </c>
+      <c r="CL53" t="n">
+        <v>105.8</v>
+      </c>
+      <c r="CM53" t="n">
+        <v>104.9</v>
+      </c>
+      <c r="CN53" t="n">
+        <v>104.9</v>
+      </c>
+      <c r="CO53" t="n">
+        <v>80.5</v>
+      </c>
+      <c r="CP53" t="n">
+        <v>81.59999999999999</v>
+      </c>
+      <c r="CQ53" t="n">
+        <v>109.1</v>
+      </c>
+      <c r="CR53" t="n">
+        <v>107.6</v>
+      </c>
+      <c r="CS53" t="n">
+        <v>109</v>
+      </c>
+      <c r="CT53" t="n">
+        <v>109.4</v>
+      </c>
+      <c r="CU53" t="n">
+        <v>106.5</v>
+      </c>
+      <c r="CV53" t="n">
+        <v>85.5</v>
+      </c>
+      <c r="CW53" t="n">
+        <v>51.3</v>
+      </c>
+      <c r="CX53" t="n">
+        <v>110.6</v>
+      </c>
+      <c r="CY53" t="n">
+        <v>108</v>
+      </c>
+      <c r="CZ53" t="n">
+        <v>103.15</v>
+      </c>
+      <c r="DA53" t="n">
+        <v>111.8</v>
+      </c>
+      <c r="DB53" t="n">
+        <v>109.8</v>
+      </c>
+      <c r="DC53" t="n">
+        <v>107.6</v>
+      </c>
+      <c r="DD53" t="n">
+        <v>107.8</v>
+      </c>
+      <c r="DE53" t="n">
+        <v>109.55</v>
+      </c>
+      <c r="DF53" t="n">
+        <v>111.65</v>
+      </c>
+      <c r="DG53" t="n">
+        <v>102.65</v>
+      </c>
+      <c r="DH53" t="n">
+        <v>109.1</v>
+      </c>
+      <c r="DI53" t="n">
+        <v>112.8</v>
+      </c>
+      <c r="DJ53" t="n">
+        <v>109.4</v>
+      </c>
+      <c r="DK53" t="n">
+        <v>110.8</v>
+      </c>
+      <c r="DL53" t="n">
+        <v>108.6</v>
+      </c>
+      <c r="DM53" t="n">
+        <v>111.8</v>
+      </c>
+      <c r="DO53" t="n">
+        <v>109.95</v>
+      </c>
+      <c r="DP53" t="n">
+        <v>93.37</v>
+      </c>
+      <c r="DQ53" t="n">
+        <v>114.3</v>
+      </c>
+      <c r="DR53" t="n">
+        <v>107.95</v>
+      </c>
+      <c r="DS53" t="n">
+        <v>110.55</v>
+      </c>
+      <c r="DT53" t="n">
+        <v>111.25</v>
+      </c>
+      <c r="DU53" t="n">
+        <v>106.25</v>
+      </c>
+      <c r="DV53" t="n">
+        <v>106.6</v>
+      </c>
+      <c r="DW53" t="n">
+        <v>106.4</v>
+      </c>
+      <c r="DX53" t="n">
+        <v>108.45</v>
+      </c>
+      <c r="DY53" t="n">
+        <v>110.3</v>
+      </c>
+      <c r="DZ53" t="n">
+        <v>108.1</v>
+      </c>
+      <c r="EA53" t="n">
+        <v>108.95</v>
+      </c>
+      <c r="EB53" t="n">
+        <v>110.3</v>
+      </c>
+      <c r="EC53" t="n">
+        <v>103.95</v>
+      </c>
+      <c r="ED53" t="n">
+        <v>106.2</v>
+      </c>
+      <c r="EE53" t="n">
+        <v>103.85</v>
+      </c>
+      <c r="EF53" t="n">
+        <v>105.8</v>
+      </c>
+      <c r="EG53" t="n">
+        <v>107.85</v>
+      </c>
+      <c r="EH53" t="n">
+        <v>110.4</v>
+      </c>
+      <c r="EI53" t="n">
+        <v>104.35</v>
+      </c>
+      <c r="EJ53" t="n">
+        <v>103.75</v>
+      </c>
+      <c r="EK53" t="n">
+        <v>104.1</v>
+      </c>
+      <c r="EL53" t="n">
+        <v>106.05</v>
+      </c>
+      <c r="EM53" t="n">
+        <v>101.55</v>
+      </c>
+      <c r="EN53" t="n">
+        <v>112</v>
+      </c>
+      <c r="EO53" t="n">
+        <v>103.65</v>
+      </c>
+      <c r="EP53" t="n">
+        <v>103.2</v>
+      </c>
+      <c r="EQ53" t="n">
+        <v>103.5</v>
+      </c>
+      <c r="ER53" t="n">
+        <v>104.4</v>
+      </c>
+      <c r="ES53" t="n">
+        <v>102</v>
+      </c>
+      <c r="ET53" t="n">
+        <v>101.7</v>
+      </c>
+      <c r="EU53" t="n">
+        <v>104</v>
+      </c>
+      <c r="EV53" t="n">
+        <v>101.8</v>
+      </c>
+      <c r="EW53" t="n">
+        <v>102.75</v>
+      </c>
+      <c r="EX53" t="n">
+        <v>103.4</v>
+      </c>
+      <c r="EY53" t="n">
+        <v>109.85</v>
+      </c>
+      <c r="EZ53" t="n">
+        <v>102.2</v>
+      </c>
+      <c r="FA53" t="n">
+        <v>103.4</v>
+      </c>
+      <c r="FB53" t="n">
+        <v>103.75</v>
+      </c>
+      <c r="FC53" t="n">
+        <v>105.4</v>
+      </c>
+      <c r="FD53" t="n">
+        <v>100</v>
+      </c>
+      <c r="FE53" t="n">
+        <v>105.5</v>
+      </c>
+      <c r="FF53" t="n">
+        <v>104</v>
+      </c>
+      <c r="FH53" t="n">
+        <v>105.8</v>
+      </c>
+      <c r="FI53" t="n">
+        <v>104.9</v>
+      </c>
+      <c r="FJ53" t="n">
+        <v>102.1</v>
+      </c>
+      <c r="FK53" t="n">
+        <v>102.8</v>
+      </c>
+      <c r="FL53" t="n">
+        <v>101.75</v>
+      </c>
+      <c r="FM53" t="n">
+        <v>104.05</v>
+      </c>
+      <c r="FN53" t="n">
+        <v>106</v>
+      </c>
       <c r="FQ53" t="n">
         <v>100.369</v>
       </c>
@@ -25041,6 +25299,21 @@
       </c>
       <c r="FS53" t="n">
         <v>136700</v>
+      </c>
+      <c r="FU53" t="n">
+        <v>100.4</v>
+      </c>
+      <c r="FV53" t="n">
+        <v>99.98999999999999</v>
+      </c>
+      <c r="FW53" t="n">
+        <v>102</v>
+      </c>
+      <c r="FX53" t="n">
+        <v>103</v>
+      </c>
+      <c r="FY53" t="n">
+        <v>25.95</v>
       </c>
       <c r="FZ53" t="n">
         <v>110.85</v>
@@ -27732,6 +28005,18 @@
       <c r="BK59" t="n">
         <v>146700</v>
       </c>
+      <c r="BM59" t="n">
+        <v>101.2</v>
+      </c>
+      <c r="BN59" t="n">
+        <v>108.7</v>
+      </c>
+      <c r="BO59" t="n">
+        <v>114.1</v>
+      </c>
+      <c r="BP59" t="n">
+        <v>108.2</v>
+      </c>
       <c r="BQ59" t="n">
         <v>148400</v>
       </c>
@@ -27780,11 +28065,281 @@
       <c r="CG59" t="n">
         <v>102.6</v>
       </c>
+      <c r="CH59" t="n">
+        <v>47.99999999999999</v>
+      </c>
+      <c r="CI59" t="n">
+        <v>64.34999999999999</v>
+      </c>
+      <c r="CJ59" t="n">
+        <v>112.4</v>
+      </c>
+      <c r="CL59" t="n">
+        <v>105.95</v>
+      </c>
+      <c r="CM59" t="n">
+        <v>104.75</v>
+      </c>
+      <c r="CN59" t="n">
+        <v>105</v>
+      </c>
+      <c r="CO59" t="n">
+        <v>78.40000000000001</v>
+      </c>
+      <c r="CP59" t="n">
+        <v>79.5</v>
+      </c>
+      <c r="CQ59" t="n">
+        <v>109.75</v>
+      </c>
+      <c r="CR59" t="n">
+        <v>108.75</v>
+      </c>
+      <c r="CS59" t="n">
+        <v>109.95</v>
+      </c>
+      <c r="CT59" t="n">
+        <v>109.85</v>
+      </c>
+      <c r="CU59" t="n">
+        <v>106.95</v>
+      </c>
+      <c r="CV59" t="n">
+        <v>84.62</v>
+      </c>
+      <c r="CW59" t="n">
+        <v>51.46999999999998</v>
+      </c>
+      <c r="CX59" t="n">
+        <v>110.45</v>
+      </c>
+      <c r="CY59" t="n">
+        <v>107.8</v>
+      </c>
+      <c r="CZ59" t="n">
+        <v>104</v>
+      </c>
+      <c r="DA59" t="n">
+        <v>112.35</v>
+      </c>
+      <c r="DB59" t="n">
+        <v>110.5</v>
+      </c>
+      <c r="DC59" t="n">
+        <v>107.45</v>
+      </c>
+      <c r="DD59" t="n">
+        <v>107.65</v>
+      </c>
+      <c r="DE59" t="n">
+        <v>110.2</v>
+      </c>
+      <c r="DF59" t="n">
+        <v>111.35</v>
+      </c>
+      <c r="DG59" t="n">
+        <v>104.4</v>
+      </c>
+      <c r="DH59" t="n">
+        <v>109</v>
+      </c>
+      <c r="DI59" t="n">
+        <v>113</v>
+      </c>
+      <c r="DJ59" t="n">
+        <v>109.75</v>
+      </c>
+      <c r="DK59" t="n">
+        <v>111.3</v>
+      </c>
+      <c r="DL59" t="n">
+        <v>109.3</v>
+      </c>
+      <c r="DM59" t="n">
+        <v>112.3</v>
+      </c>
+      <c r="DN59" t="n">
+        <v>109.2</v>
+      </c>
+      <c r="DO59" t="n">
+        <v>110</v>
+      </c>
+      <c r="DP59" t="n">
+        <v>93.55</v>
+      </c>
+      <c r="DQ59" t="n">
+        <v>114.3</v>
+      </c>
+      <c r="DR59" t="n">
+        <v>107.95</v>
+      </c>
+      <c r="DS59" t="n">
+        <v>110.85</v>
+      </c>
+      <c r="DT59" t="n">
+        <v>110.9</v>
+      </c>
+      <c r="DU59" t="n">
+        <v>106.05</v>
+      </c>
+      <c r="DV59" t="n">
+        <v>106.8</v>
+      </c>
+      <c r="DW59" t="n">
+        <v>108</v>
+      </c>
+      <c r="DX59" t="n">
+        <v>105.3</v>
+      </c>
+      <c r="DY59" t="n">
+        <v>110.25</v>
+      </c>
+      <c r="DZ59" t="n">
+        <v>108.1</v>
+      </c>
+      <c r="EA59" t="n">
+        <v>108.6</v>
+      </c>
+      <c r="EB59" t="n">
+        <v>106.4</v>
+      </c>
+      <c r="EC59" t="n">
+        <v>103.1</v>
+      </c>
+      <c r="ED59" t="n">
+        <v>106.85</v>
+      </c>
+      <c r="EE59" t="n">
+        <v>103.2</v>
+      </c>
+      <c r="EF59" t="n">
+        <v>106.35</v>
+      </c>
+      <c r="EG59" t="n">
+        <v>108.25</v>
+      </c>
+      <c r="EH59" t="n">
+        <v>111.7</v>
+      </c>
+      <c r="EI59" t="n">
+        <v>101.95</v>
+      </c>
+      <c r="EJ59" t="n">
+        <v>103.7</v>
+      </c>
+      <c r="EK59" t="n">
+        <v>103.8</v>
+      </c>
+      <c r="EL59" t="n">
+        <v>105.9</v>
+      </c>
+      <c r="EM59" t="n">
+        <v>101.35</v>
+      </c>
+      <c r="EN59" t="n">
+        <v>111.7</v>
+      </c>
+      <c r="EO59" t="n">
+        <v>103.4</v>
+      </c>
+      <c r="EQ59" t="n">
+        <v>104.45</v>
+      </c>
+      <c r="ER59" t="n">
+        <v>103.8</v>
+      </c>
+      <c r="ES59" t="n">
+        <v>102</v>
+      </c>
+      <c r="ET59" t="n">
+        <v>101.65</v>
+      </c>
+      <c r="EU59" t="n">
+        <v>104.05</v>
+      </c>
+      <c r="EV59" t="n">
+        <v>103.45</v>
+      </c>
+      <c r="EW59" t="n">
+        <v>102.8</v>
+      </c>
+      <c r="EX59" t="n">
+        <v>105.5</v>
+      </c>
+      <c r="EY59" t="n">
+        <v>111.8</v>
+      </c>
+      <c r="EZ59" t="n">
+        <v>102</v>
+      </c>
+      <c r="FA59" t="n">
+        <v>103.9</v>
+      </c>
+      <c r="FB59" t="n">
+        <v>103.5</v>
+      </c>
+      <c r="FC59" t="n">
+        <v>104.9</v>
+      </c>
+      <c r="FD59" t="n">
+        <v>99.99999999999999</v>
+      </c>
+      <c r="FE59" t="n">
+        <v>105.75</v>
+      </c>
+      <c r="FF59" t="n">
+        <v>103.9</v>
+      </c>
+      <c r="FG59" t="n">
+        <v>100.4</v>
+      </c>
+      <c r="FH59" t="n">
+        <v>105.65</v>
+      </c>
+      <c r="FI59" t="n">
+        <v>104.5</v>
+      </c>
+      <c r="FJ59" t="n">
+        <v>101.8</v>
+      </c>
+      <c r="FK59" t="n">
+        <v>102.8</v>
+      </c>
+      <c r="FL59" t="n">
+        <v>102.4</v>
+      </c>
+      <c r="FM59" t="n">
+        <v>104.4</v>
+      </c>
+      <c r="FN59" t="n">
+        <v>106.2</v>
+      </c>
       <c r="FQ59" t="n">
         <v>100.9</v>
       </c>
       <c r="FS59" t="n">
         <v>136890</v>
+      </c>
+      <c r="FU59" t="n">
+        <v>100.45</v>
+      </c>
+      <c r="FV59" t="n">
+        <v>100.3</v>
+      </c>
+      <c r="FX59" t="n">
+        <v>103.65</v>
+      </c>
+      <c r="FY59" t="n">
+        <v>25.85</v>
+      </c>
+      <c r="FZ59" t="n">
+        <v>111.75</v>
+      </c>
+      <c r="GA59" t="n">
+        <v>104.5</v>
+      </c>
+      <c r="GB59" t="n">
+        <v>100.85</v>
       </c>
     </row>
     <row r="60">
@@ -28448,6 +29003,18 @@
       <c r="BK61" t="n">
         <v>145600</v>
       </c>
+      <c r="BM61" t="n">
+        <v>101.5</v>
+      </c>
+      <c r="BN61" t="n">
+        <v>106.25</v>
+      </c>
+      <c r="BO61" t="n">
+        <v>113.85</v>
+      </c>
+      <c r="BP61" t="n">
+        <v>108.55</v>
+      </c>
       <c r="BQ61" t="n">
         <v>148380</v>
       </c>
@@ -28496,11 +29063,278 @@
       <c r="CG61" t="n">
         <v>102.8</v>
       </c>
+      <c r="CH61" t="n">
+        <v>48.35</v>
+      </c>
+      <c r="CI61" t="n">
+        <v>64.2</v>
+      </c>
+      <c r="CJ61" t="n">
+        <v>111.75</v>
+      </c>
+      <c r="CL61" t="n">
+        <v>106.5</v>
+      </c>
+      <c r="CM61" t="n">
+        <v>104.55</v>
+      </c>
+      <c r="CN61" t="n">
+        <v>105.45</v>
+      </c>
+      <c r="CO61" t="n">
+        <v>78.04000000000001</v>
+      </c>
+      <c r="CP61" t="n">
+        <v>79.79000000000001</v>
+      </c>
+      <c r="CQ61" t="n">
+        <v>110</v>
+      </c>
+      <c r="CR61" t="n">
+        <v>108.6</v>
+      </c>
+      <c r="CS61" t="n">
+        <v>110.25</v>
+      </c>
+      <c r="CT61" t="n">
+        <v>110.2</v>
+      </c>
+      <c r="CU61" t="n">
+        <v>107</v>
+      </c>
+      <c r="CV61" t="n">
+        <v>84.26000000000001</v>
+      </c>
+      <c r="CW61" t="n">
+        <v>51.66</v>
+      </c>
+      <c r="CX61" t="n">
+        <v>110.7</v>
+      </c>
+      <c r="CY61" t="n">
+        <v>108.25</v>
+      </c>
+      <c r="CZ61" t="n">
+        <v>104.2</v>
+      </c>
+      <c r="DA61" t="n">
+        <v>112.5</v>
+      </c>
+      <c r="DB61" t="n">
+        <v>109.85</v>
+      </c>
+      <c r="DC61" t="n">
+        <v>107.8</v>
+      </c>
+      <c r="DD61" t="n">
+        <v>108.2</v>
+      </c>
+      <c r="DE61" t="n">
+        <v>110.7</v>
+      </c>
+      <c r="DF61" t="n">
+        <v>111.4</v>
+      </c>
+      <c r="DG61" t="n">
+        <v>104.7</v>
+      </c>
+      <c r="DH61" t="n">
+        <v>108.95</v>
+      </c>
+      <c r="DI61" t="n">
+        <v>113.4</v>
+      </c>
+      <c r="DJ61" t="n">
+        <v>110.4</v>
+      </c>
+      <c r="DK61" t="n">
+        <v>111</v>
+      </c>
+      <c r="DL61" t="n">
+        <v>109.8</v>
+      </c>
+      <c r="DM61" t="n">
+        <v>112.6</v>
+      </c>
+      <c r="DN61" t="n">
+        <v>109</v>
+      </c>
+      <c r="DO61" t="n">
+        <v>110.3</v>
+      </c>
+      <c r="DP61" t="n">
+        <v>93.75</v>
+      </c>
+      <c r="DQ61" t="n">
+        <v>114.2</v>
+      </c>
+      <c r="DR61" t="n">
+        <v>107.85</v>
+      </c>
+      <c r="DS61" t="n">
+        <v>111.1</v>
+      </c>
+      <c r="DT61" t="n">
+        <v>110.75</v>
+      </c>
+      <c r="DU61" t="n">
+        <v>106.7</v>
+      </c>
+      <c r="DV61" t="n">
+        <v>107</v>
+      </c>
+      <c r="DW61" t="n">
+        <v>106.5</v>
+      </c>
+      <c r="DX61" t="n">
+        <v>105.4</v>
+      </c>
+      <c r="DY61" t="n">
+        <v>110.55</v>
+      </c>
+      <c r="DZ61" t="n">
+        <v>107.85</v>
+      </c>
+      <c r="EA61" t="n">
+        <v>109.7</v>
+      </c>
+      <c r="EB61" t="n">
+        <v>106.1</v>
+      </c>
+      <c r="EC61" t="n">
+        <v>103.7</v>
+      </c>
+      <c r="ED61" t="n">
+        <v>106.25</v>
+      </c>
+      <c r="EE61" t="n">
+        <v>102.85</v>
+      </c>
+      <c r="EF61" t="n">
+        <v>106.05</v>
+      </c>
+      <c r="EG61" t="n">
+        <v>107.8</v>
+      </c>
+      <c r="EH61" t="n">
+        <v>111.5</v>
+      </c>
+      <c r="EI61" t="n">
+        <v>101.95</v>
+      </c>
+      <c r="EJ61" t="n">
+        <v>103.6</v>
+      </c>
+      <c r="EK61" t="n">
+        <v>103.65</v>
+      </c>
+      <c r="EL61" t="n">
+        <v>106.5</v>
+      </c>
+      <c r="EM61" t="n">
+        <v>101.2</v>
+      </c>
+      <c r="EN61" t="n">
+        <v>111.85</v>
+      </c>
+      <c r="EQ61" t="n">
+        <v>104</v>
+      </c>
+      <c r="ER61" t="n">
+        <v>103.75</v>
+      </c>
+      <c r="ES61" t="n">
+        <v>102</v>
+      </c>
+      <c r="ET61" t="n">
+        <v>101.7</v>
+      </c>
+      <c r="EU61" t="n">
+        <v>104</v>
+      </c>
+      <c r="EV61" t="n">
+        <v>102.5</v>
+      </c>
+      <c r="EW61" t="n">
+        <v>103</v>
+      </c>
+      <c r="EX61" t="n">
+        <v>107</v>
+      </c>
+      <c r="EY61" t="n">
+        <v>110.95</v>
+      </c>
+      <c r="EZ61" t="n">
+        <v>102.1</v>
+      </c>
+      <c r="FA61" t="n">
+        <v>103.6</v>
+      </c>
+      <c r="FB61" t="n">
+        <v>103.8</v>
+      </c>
+      <c r="FC61" t="n">
+        <v>105.1</v>
+      </c>
+      <c r="FD61" t="n">
+        <v>99.98999999999999</v>
+      </c>
+      <c r="FE61" t="n">
+        <v>105.5</v>
+      </c>
+      <c r="FF61" t="n">
+        <v>104.45</v>
+      </c>
+      <c r="FG61" t="n">
+        <v>100.45</v>
+      </c>
+      <c r="FH61" t="n">
+        <v>105.75</v>
+      </c>
+      <c r="FI61" t="n">
+        <v>104.4</v>
+      </c>
+      <c r="FJ61" t="n">
+        <v>103</v>
+      </c>
+      <c r="FK61" t="n">
+        <v>103.1</v>
+      </c>
+      <c r="FL61" t="n">
+        <v>102.25</v>
+      </c>
+      <c r="FM61" t="n">
+        <v>104.7</v>
+      </c>
+      <c r="FN61" t="n">
+        <v>104.9</v>
+      </c>
       <c r="FQ61" t="n">
         <v>101.18</v>
       </c>
       <c r="FS61" t="n">
         <v>136740</v>
+      </c>
+      <c r="FU61" t="n">
+        <v>99.59999999999998</v>
+      </c>
+      <c r="FV61" t="n">
+        <v>99.95</v>
+      </c>
+      <c r="FX61" t="n">
+        <v>103.95</v>
+      </c>
+      <c r="FY61" t="n">
+        <v>25.80099999999999</v>
+      </c>
+      <c r="FZ61" t="n">
+        <v>112.5</v>
+      </c>
+      <c r="GA61" t="n">
+        <v>105.5</v>
+      </c>
+      <c r="GB61" t="n">
+        <v>101</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Rellenar historia de instrumentos nuevos 2026-08-19
</commit_message>
<xml_diff>
--- a/historicos.xlsx
+++ b/historicos.xlsx
@@ -1800,6 +1800,21 @@
       <c r="FM2" t="n">
         <v>103.9</v>
       </c>
+      <c r="GE2" t="n">
+        <v>109</v>
+      </c>
+      <c r="GF2" t="n">
+        <v>103.6</v>
+      </c>
+      <c r="GH2" t="n">
+        <v>106.35</v>
+      </c>
+      <c r="GJ2" t="n">
+        <v>101.5</v>
+      </c>
+      <c r="GK2" t="n">
+        <v>106.5</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -2230,6 +2245,27 @@
       <c r="FZ3" t="n">
         <v>108.8</v>
       </c>
+      <c r="GE3" t="n">
+        <v>112.8</v>
+      </c>
+      <c r="GF3" t="n">
+        <v>105.15</v>
+      </c>
+      <c r="GG3" t="n">
+        <v>103.4</v>
+      </c>
+      <c r="GH3" t="n">
+        <v>106.2</v>
+      </c>
+      <c r="GI3" t="n">
+        <v>105</v>
+      </c>
+      <c r="GJ3" t="n">
+        <v>102.25</v>
+      </c>
+      <c r="GK3" t="n">
+        <v>105.8</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -2660,6 +2696,27 @@
       <c r="FZ4" t="n">
         <v>108.45</v>
       </c>
+      <c r="GE4" t="n">
+        <v>112.9</v>
+      </c>
+      <c r="GF4" t="n">
+        <v>105</v>
+      </c>
+      <c r="GG4" t="n">
+        <v>102.9</v>
+      </c>
+      <c r="GH4" t="n">
+        <v>105.75</v>
+      </c>
+      <c r="GI4" t="n">
+        <v>106.75</v>
+      </c>
+      <c r="GJ4" t="n">
+        <v>102.2</v>
+      </c>
+      <c r="GK4" t="n">
+        <v>105.4</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -3093,6 +3150,27 @@
       <c r="FZ5" t="n">
         <v>108.4</v>
       </c>
+      <c r="GE5" t="n">
+        <v>112.7</v>
+      </c>
+      <c r="GF5" t="n">
+        <v>104.75</v>
+      </c>
+      <c r="GG5" t="n">
+        <v>102.9</v>
+      </c>
+      <c r="GH5" t="n">
+        <v>105.7</v>
+      </c>
+      <c r="GI5" t="n">
+        <v>104.7</v>
+      </c>
+      <c r="GJ5" t="n">
+        <v>102.85</v>
+      </c>
+      <c r="GK5" t="n">
+        <v>105</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -3541,6 +3619,27 @@
       <c r="FZ6" t="n">
         <v>109</v>
       </c>
+      <c r="GE6" t="n">
+        <v>112.2</v>
+      </c>
+      <c r="GF6" t="n">
+        <v>104</v>
+      </c>
+      <c r="GG6" t="n">
+        <v>103.75</v>
+      </c>
+      <c r="GH6" t="n">
+        <v>105.85</v>
+      </c>
+      <c r="GI6" t="n">
+        <v>105.05</v>
+      </c>
+      <c r="GJ6" t="n">
+        <v>102.65</v>
+      </c>
+      <c r="GK6" t="n">
+        <v>105.75</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -4001,6 +4100,27 @@
       <c r="FZ7" t="n">
         <v>109</v>
       </c>
+      <c r="GE7" t="n">
+        <v>112.35</v>
+      </c>
+      <c r="GF7" t="n">
+        <v>104</v>
+      </c>
+      <c r="GG7" t="n">
+        <v>104</v>
+      </c>
+      <c r="GH7" t="n">
+        <v>105.9</v>
+      </c>
+      <c r="GI7" t="n">
+        <v>105.5</v>
+      </c>
+      <c r="GJ7" t="n">
+        <v>102</v>
+      </c>
+      <c r="GK7" t="n">
+        <v>105.15</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -4455,6 +4575,27 @@
       <c r="FZ8" t="n">
         <v>109</v>
       </c>
+      <c r="GE8" t="n">
+        <v>112.6</v>
+      </c>
+      <c r="GF8" t="n">
+        <v>103.7</v>
+      </c>
+      <c r="GG8" t="n">
+        <v>104</v>
+      </c>
+      <c r="GH8" t="n">
+        <v>106.1</v>
+      </c>
+      <c r="GI8" t="n">
+        <v>104.95</v>
+      </c>
+      <c r="GJ8" t="n">
+        <v>102.7</v>
+      </c>
+      <c r="GK8" t="n">
+        <v>107</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -4915,6 +5056,27 @@
       <c r="FZ9" t="n">
         <v>110</v>
       </c>
+      <c r="GE9" t="n">
+        <v>112.85</v>
+      </c>
+      <c r="GF9" t="n">
+        <v>103.7</v>
+      </c>
+      <c r="GG9" t="n">
+        <v>103.8</v>
+      </c>
+      <c r="GH9" t="n">
+        <v>106.1</v>
+      </c>
+      <c r="GI9" t="n">
+        <v>104.8</v>
+      </c>
+      <c r="GJ9" t="n">
+        <v>102.4</v>
+      </c>
+      <c r="GK9" t="n">
+        <v>105.55</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -5378,6 +5540,27 @@
       <c r="FZ10" t="n">
         <v>110.2</v>
       </c>
+      <c r="GE10" t="n">
+        <v>112.8</v>
+      </c>
+      <c r="GF10" t="n">
+        <v>103.75</v>
+      </c>
+      <c r="GG10" t="n">
+        <v>105.85</v>
+      </c>
+      <c r="GH10" t="n">
+        <v>106.1</v>
+      </c>
+      <c r="GI10" t="n">
+        <v>105.2</v>
+      </c>
+      <c r="GJ10" t="n">
+        <v>102.1</v>
+      </c>
+      <c r="GK10" t="n">
+        <v>105.5</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -5829,6 +6012,27 @@
       <c r="FN11" t="n">
         <v>101.5</v>
       </c>
+      <c r="GE11" t="n">
+        <v>112.65</v>
+      </c>
+      <c r="GF11" t="n">
+        <v>104</v>
+      </c>
+      <c r="GG11" t="n">
+        <v>105.9</v>
+      </c>
+      <c r="GH11" t="n">
+        <v>106.25</v>
+      </c>
+      <c r="GI11" t="n">
+        <v>104.15</v>
+      </c>
+      <c r="GJ11" t="n">
+        <v>102.7</v>
+      </c>
+      <c r="GK11" t="n">
+        <v>104.65</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -6277,6 +6481,27 @@
       <c r="FN12" t="n">
         <v>102.25</v>
       </c>
+      <c r="GE12" t="n">
+        <v>113</v>
+      </c>
+      <c r="GF12" t="n">
+        <v>104.2</v>
+      </c>
+      <c r="GG12" t="n">
+        <v>102.5</v>
+      </c>
+      <c r="GH12" t="n">
+        <v>106.4</v>
+      </c>
+      <c r="GI12" t="n">
+        <v>104.6</v>
+      </c>
+      <c r="GJ12" t="n">
+        <v>102.45</v>
+      </c>
+      <c r="GK12" t="n">
+        <v>105.25</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -6740,6 +6965,27 @@
       <c r="FZ13" t="n">
         <v>111.65</v>
       </c>
+      <c r="GE13" t="n">
+        <v>113.65</v>
+      </c>
+      <c r="GF13" t="n">
+        <v>104.85</v>
+      </c>
+      <c r="GG13" t="n">
+        <v>102.5</v>
+      </c>
+      <c r="GH13" t="n">
+        <v>106.7</v>
+      </c>
+      <c r="GI13" t="n">
+        <v>105.2</v>
+      </c>
+      <c r="GJ13" t="n">
+        <v>103.1</v>
+      </c>
+      <c r="GK13" t="n">
+        <v>105.25</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -7203,6 +7449,27 @@
       <c r="FZ14" t="n">
         <v>110</v>
       </c>
+      <c r="GE14" t="n">
+        <v>113.35</v>
+      </c>
+      <c r="GF14" t="n">
+        <v>104.95</v>
+      </c>
+      <c r="GG14" t="n">
+        <v>101.9</v>
+      </c>
+      <c r="GH14" t="n">
+        <v>106.6</v>
+      </c>
+      <c r="GI14" t="n">
+        <v>105.4</v>
+      </c>
+      <c r="GJ14" t="n">
+        <v>102.7</v>
+      </c>
+      <c r="GK14" t="n">
+        <v>105.8</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -7654,6 +7921,30 @@
       <c r="FO15" t="n">
         <v>98.75</v>
       </c>
+      <c r="FW15" t="n">
+        <v>99</v>
+      </c>
+      <c r="GE15" t="n">
+        <v>112.7</v>
+      </c>
+      <c r="GF15" t="n">
+        <v>104.8</v>
+      </c>
+      <c r="GG15" t="n">
+        <v>102.3</v>
+      </c>
+      <c r="GH15" t="n">
+        <v>106.5</v>
+      </c>
+      <c r="GI15" t="n">
+        <v>105.5</v>
+      </c>
+      <c r="GJ15" t="n">
+        <v>102.6</v>
+      </c>
+      <c r="GK15" t="n">
+        <v>105.85</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -8123,8 +8414,32 @@
       <c r="FN16" t="n">
         <v>102.75</v>
       </c>
+      <c r="FW16" t="n">
+        <v>99.20000000000002</v>
+      </c>
       <c r="FZ16" t="n">
         <v>112.55</v>
+      </c>
+      <c r="GE16" t="n">
+        <v>112.55</v>
+      </c>
+      <c r="GF16" t="n">
+        <v>105.8</v>
+      </c>
+      <c r="GG16" t="n">
+        <v>103.2</v>
+      </c>
+      <c r="GH16" t="n">
+        <v>107</v>
+      </c>
+      <c r="GI16" t="n">
+        <v>105.2</v>
+      </c>
+      <c r="GJ16" t="n">
+        <v>102.4</v>
+      </c>
+      <c r="GK16" t="n">
+        <v>105.9</v>
       </c>
     </row>
     <row r="17">
@@ -8592,8 +8907,32 @@
       <c r="FN17" t="n">
         <v>102.7</v>
       </c>
+      <c r="FW17" t="n">
+        <v>100</v>
+      </c>
       <c r="FZ17" t="n">
         <v>113.5</v>
+      </c>
+      <c r="GE17" t="n">
+        <v>112.45</v>
+      </c>
+      <c r="GF17" t="n">
+        <v>105.2</v>
+      </c>
+      <c r="GG17" t="n">
+        <v>102.75</v>
+      </c>
+      <c r="GH17" t="n">
+        <v>106.75</v>
+      </c>
+      <c r="GI17" t="n">
+        <v>105.75</v>
+      </c>
+      <c r="GJ17" t="n">
+        <v>102.4</v>
+      </c>
+      <c r="GK17" t="n">
+        <v>105.85</v>
       </c>
     </row>
     <row r="18">
@@ -9058,6 +9397,30 @@
       <c r="FN18" t="n">
         <v>102.75</v>
       </c>
+      <c r="FW18" t="n">
+        <v>100.5</v>
+      </c>
+      <c r="GE18" t="n">
+        <v>112.15</v>
+      </c>
+      <c r="GF18" t="n">
+        <v>104.9</v>
+      </c>
+      <c r="GG18" t="n">
+        <v>103.7</v>
+      </c>
+      <c r="GH18" t="n">
+        <v>106.65</v>
+      </c>
+      <c r="GI18" t="n">
+        <v>105</v>
+      </c>
+      <c r="GJ18" t="n">
+        <v>102.5</v>
+      </c>
+      <c r="GK18" t="n">
+        <v>106</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -9530,6 +9893,30 @@
       <c r="FN19" t="n">
         <v>102.75</v>
       </c>
+      <c r="FW19" t="n">
+        <v>100.5</v>
+      </c>
+      <c r="GE19" t="n">
+        <v>112.55</v>
+      </c>
+      <c r="GF19" t="n">
+        <v>105.95</v>
+      </c>
+      <c r="GG19" t="n">
+        <v>102.75</v>
+      </c>
+      <c r="GH19" t="n">
+        <v>106.65</v>
+      </c>
+      <c r="GI19" t="n">
+        <v>106</v>
+      </c>
+      <c r="GJ19" t="n">
+        <v>102.6</v>
+      </c>
+      <c r="GK19" t="n">
+        <v>105.9</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -9996,8 +10383,32 @@
       <c r="FN20" t="n">
         <v>102.6</v>
       </c>
+      <c r="FW20" t="n">
+        <v>100.5</v>
+      </c>
       <c r="FZ20" t="n">
         <v>113</v>
+      </c>
+      <c r="GE20" t="n">
+        <v>112.35</v>
+      </c>
+      <c r="GF20" t="n">
+        <v>105.2</v>
+      </c>
+      <c r="GG20" t="n">
+        <v>102.8</v>
+      </c>
+      <c r="GH20" t="n">
+        <v>107.05</v>
+      </c>
+      <c r="GI20" t="n">
+        <v>105.9</v>
+      </c>
+      <c r="GJ20" t="n">
+        <v>102.7</v>
+      </c>
+      <c r="GK20" t="n">
+        <v>105.95</v>
       </c>
     </row>
     <row r="21">
@@ -10468,6 +10879,30 @@
       <c r="FN21" t="n">
         <v>102</v>
       </c>
+      <c r="FW21" t="n">
+        <v>100.3</v>
+      </c>
+      <c r="GE21" t="n">
+        <v>111.9</v>
+      </c>
+      <c r="GF21" t="n">
+        <v>104.75</v>
+      </c>
+      <c r="GG21" t="n">
+        <v>103.5</v>
+      </c>
+      <c r="GH21" t="n">
+        <v>106.7</v>
+      </c>
+      <c r="GI21" t="n">
+        <v>105.4</v>
+      </c>
+      <c r="GJ21" t="n">
+        <v>102.5</v>
+      </c>
+      <c r="GK21" t="n">
+        <v>105.95</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -10940,8 +11375,35 @@
       <c r="FN22" t="n">
         <v>102.5</v>
       </c>
+      <c r="FT22" t="n">
+        <v>95</v>
+      </c>
+      <c r="FW22" t="n">
+        <v>100.15</v>
+      </c>
       <c r="FZ22" t="n">
         <v>112.55</v>
+      </c>
+      <c r="GE22" t="n">
+        <v>112.2</v>
+      </c>
+      <c r="GF22" t="n">
+        <v>105.6</v>
+      </c>
+      <c r="GG22" t="n">
+        <v>103.25</v>
+      </c>
+      <c r="GH22" t="n">
+        <v>106.55</v>
+      </c>
+      <c r="GI22" t="n">
+        <v>105.25</v>
+      </c>
+      <c r="GJ22" t="n">
+        <v>102.35</v>
+      </c>
+      <c r="GK22" t="n">
+        <v>106.3</v>
       </c>
     </row>
     <row r="23">
@@ -11412,8 +11874,32 @@
       <c r="FN23" t="n">
         <v>102.7</v>
       </c>
+      <c r="FW23" t="n">
+        <v>100.5</v>
+      </c>
       <c r="FZ23" t="n">
         <v>112.55</v>
+      </c>
+      <c r="GE23" t="n">
+        <v>112</v>
+      </c>
+      <c r="GF23" t="n">
+        <v>104.65</v>
+      </c>
+      <c r="GG23" t="n">
+        <v>103</v>
+      </c>
+      <c r="GH23" t="n">
+        <v>106.6</v>
+      </c>
+      <c r="GI23" t="n">
+        <v>105.7</v>
+      </c>
+      <c r="GJ23" t="n">
+        <v>102.7</v>
+      </c>
+      <c r="GK23" t="n">
+        <v>106</v>
       </c>
     </row>
     <row r="24">
@@ -11887,8 +12373,32 @@
       <c r="FN24" t="n">
         <v>103</v>
       </c>
+      <c r="FW24" t="n">
+        <v>100.25</v>
+      </c>
       <c r="FZ24" t="n">
         <v>112.3</v>
+      </c>
+      <c r="GE24" t="n">
+        <v>112.3</v>
+      </c>
+      <c r="GF24" t="n">
+        <v>104.8</v>
+      </c>
+      <c r="GG24" t="n">
+        <v>103.8</v>
+      </c>
+      <c r="GH24" t="n">
+        <v>106.75</v>
+      </c>
+      <c r="GI24" t="n">
+        <v>105.9</v>
+      </c>
+      <c r="GJ24" t="n">
+        <v>102.55</v>
+      </c>
+      <c r="GK24" t="n">
+        <v>106</v>
       </c>
     </row>
     <row r="25">
@@ -12359,8 +12869,32 @@
       <c r="FN25" t="n">
         <v>102.9</v>
       </c>
+      <c r="FW25" t="n">
+        <v>100</v>
+      </c>
       <c r="FZ25" t="n">
         <v>112.45</v>
+      </c>
+      <c r="GE25" t="n">
+        <v>112.3</v>
+      </c>
+      <c r="GF25" t="n">
+        <v>104.6</v>
+      </c>
+      <c r="GG25" t="n">
+        <v>104</v>
+      </c>
+      <c r="GH25" t="n">
+        <v>107</v>
+      </c>
+      <c r="GI25" t="n">
+        <v>107.2</v>
+      </c>
+      <c r="GJ25" t="n">
+        <v>102.8</v>
+      </c>
+      <c r="GK25" t="n">
+        <v>104.05</v>
       </c>
     </row>
     <row r="26">
@@ -12825,8 +13359,32 @@
       <c r="FN26" t="n">
         <v>103</v>
       </c>
+      <c r="FW26" t="n">
+        <v>100.15</v>
+      </c>
       <c r="FZ26" t="n">
         <v>112.55</v>
+      </c>
+      <c r="GE26" t="n">
+        <v>112.5</v>
+      </c>
+      <c r="GF26" t="n">
+        <v>104.8</v>
+      </c>
+      <c r="GG26" t="n">
+        <v>104.5</v>
+      </c>
+      <c r="GH26" t="n">
+        <v>106.7</v>
+      </c>
+      <c r="GI26" t="n">
+        <v>106</v>
+      </c>
+      <c r="GJ26" t="n">
+        <v>102.05</v>
+      </c>
+      <c r="GK26" t="n">
+        <v>106.7</v>
       </c>
     </row>
     <row r="27">
@@ -13294,8 +13852,32 @@
       <c r="FN27" t="n">
         <v>103</v>
       </c>
+      <c r="FW27" t="n">
+        <v>100.2</v>
+      </c>
       <c r="FZ27" t="n">
         <v>112.15</v>
+      </c>
+      <c r="GE27" t="n">
+        <v>112.5</v>
+      </c>
+      <c r="GF27" t="n">
+        <v>105.5</v>
+      </c>
+      <c r="GG27" t="n">
+        <v>104.9</v>
+      </c>
+      <c r="GH27" t="n">
+        <v>107.05</v>
+      </c>
+      <c r="GI27" t="n">
+        <v>107</v>
+      </c>
+      <c r="GJ27" t="n">
+        <v>102.6</v>
+      </c>
+      <c r="GK27" t="n">
+        <v>106.7</v>
       </c>
     </row>
     <row r="28">
@@ -13769,6 +14351,30 @@
       <c r="FN28" t="n">
         <v>103</v>
       </c>
+      <c r="FW28" t="n">
+        <v>100.2</v>
+      </c>
+      <c r="GE28" t="n">
+        <v>112.2</v>
+      </c>
+      <c r="GF28" t="n">
+        <v>105.5</v>
+      </c>
+      <c r="GG28" t="n">
+        <v>103.85</v>
+      </c>
+      <c r="GH28" t="n">
+        <v>107.5</v>
+      </c>
+      <c r="GI28" t="n">
+        <v>105.8</v>
+      </c>
+      <c r="GJ28" t="n">
+        <v>103</v>
+      </c>
+      <c r="GK28" t="n">
+        <v>106.1</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -14247,8 +14853,32 @@
       <c r="FN29" t="n">
         <v>102.5</v>
       </c>
+      <c r="FW29" t="n">
+        <v>100.2</v>
+      </c>
       <c r="FZ29" t="n">
         <v>112.85</v>
+      </c>
+      <c r="GE29" t="n">
+        <v>111.85</v>
+      </c>
+      <c r="GF29" t="n">
+        <v>104.95</v>
+      </c>
+      <c r="GG29" t="n">
+        <v>104</v>
+      </c>
+      <c r="GH29" t="n">
+        <v>106.65</v>
+      </c>
+      <c r="GI29" t="n">
+        <v>106.1</v>
+      </c>
+      <c r="GJ29" t="n">
+        <v>103</v>
+      </c>
+      <c r="GK29" t="n">
+        <v>106.7</v>
       </c>
     </row>
     <row r="30">
@@ -14731,8 +15361,29 @@
       <c r="FP30" t="n">
         <v>100.1</v>
       </c>
+      <c r="FW30" t="n">
+        <v>100.6</v>
+      </c>
       <c r="FZ30" t="n">
         <v>112.8</v>
+      </c>
+      <c r="GE30" t="n">
+        <v>111.85</v>
+      </c>
+      <c r="GF30" t="n">
+        <v>105.05</v>
+      </c>
+      <c r="GG30" t="n">
+        <v>106.95</v>
+      </c>
+      <c r="GH30" t="n">
+        <v>106.7</v>
+      </c>
+      <c r="GI30" t="n">
+        <v>104.75</v>
+      </c>
+      <c r="GJ30" t="n">
+        <v>102.65</v>
       </c>
     </row>
     <row r="31">
@@ -15218,8 +15869,32 @@
       <c r="FN31" t="n">
         <v>103</v>
       </c>
+      <c r="FW31" t="n">
+        <v>100.45</v>
+      </c>
       <c r="FZ31" t="n">
         <v>112.8</v>
+      </c>
+      <c r="GE31" t="n">
+        <v>112.35</v>
+      </c>
+      <c r="GF31" t="n">
+        <v>104.9</v>
+      </c>
+      <c r="GG31" t="n">
+        <v>104.5</v>
+      </c>
+      <c r="GH31" t="n">
+        <v>107.3</v>
+      </c>
+      <c r="GI31" t="n">
+        <v>105.6</v>
+      </c>
+      <c r="GJ31" t="n">
+        <v>102.2</v>
+      </c>
+      <c r="GK31" t="n">
+        <v>102.45</v>
       </c>
     </row>
     <row r="32">
@@ -15696,8 +16371,32 @@
       <c r="FN32" t="n">
         <v>103</v>
       </c>
+      <c r="FW32" t="n">
+        <v>100.5</v>
+      </c>
       <c r="FZ32" t="n">
         <v>111.85</v>
+      </c>
+      <c r="GE32" t="n">
+        <v>112.4</v>
+      </c>
+      <c r="GF32" t="n">
+        <v>105</v>
+      </c>
+      <c r="GG32" t="n">
+        <v>105.6</v>
+      </c>
+      <c r="GH32" t="n">
+        <v>106.9</v>
+      </c>
+      <c r="GI32" t="n">
+        <v>105.7</v>
+      </c>
+      <c r="GJ32" t="n">
+        <v>102.4</v>
+      </c>
+      <c r="GK32" t="n">
+        <v>103</v>
       </c>
     </row>
     <row r="33">
@@ -16183,8 +16882,32 @@
       <c r="FN33" t="n">
         <v>103</v>
       </c>
+      <c r="FW33" t="n">
+        <v>100.9</v>
+      </c>
       <c r="FZ33" t="n">
         <v>112.8</v>
+      </c>
+      <c r="GE33" t="n">
+        <v>112.6</v>
+      </c>
+      <c r="GF33" t="n">
+        <v>105.05</v>
+      </c>
+      <c r="GG33" t="n">
+        <v>105.45</v>
+      </c>
+      <c r="GH33" t="n">
+        <v>108</v>
+      </c>
+      <c r="GI33" t="n">
+        <v>105.9</v>
+      </c>
+      <c r="GJ33" t="n">
+        <v>101.2</v>
+      </c>
+      <c r="GK33" t="n">
+        <v>102.5</v>
       </c>
     </row>
     <row r="34">
@@ -16610,6 +17333,24 @@
       <c r="FN34" t="n">
         <v>107</v>
       </c>
+      <c r="GE34" t="n">
+        <v>113</v>
+      </c>
+      <c r="GF34" t="n">
+        <v>105.6</v>
+      </c>
+      <c r="GG34" t="n">
+        <v>105.5</v>
+      </c>
+      <c r="GH34" t="n">
+        <v>107.2</v>
+      </c>
+      <c r="GJ34" t="n">
+        <v>102.4</v>
+      </c>
+      <c r="GK34" t="n">
+        <v>103</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -17097,6 +17838,27 @@
       <c r="FZ35" t="n">
         <v>112.8</v>
       </c>
+      <c r="GE35" t="n">
+        <v>112.75</v>
+      </c>
+      <c r="GF35" t="n">
+        <v>105.4</v>
+      </c>
+      <c r="GG35" t="n">
+        <v>104.75</v>
+      </c>
+      <c r="GH35" t="n">
+        <v>107</v>
+      </c>
+      <c r="GI35" t="n">
+        <v>106</v>
+      </c>
+      <c r="GJ35" t="n">
+        <v>101.95</v>
+      </c>
+      <c r="GK35" t="n">
+        <v>102.8</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -17581,8 +18343,32 @@
       <c r="FP36" t="n">
         <v>100.4</v>
       </c>
+      <c r="FW36" t="n">
+        <v>100.5</v>
+      </c>
       <c r="FZ36" t="n">
         <v>112.85</v>
+      </c>
+      <c r="GE36" t="n">
+        <v>112.1</v>
+      </c>
+      <c r="GF36" t="n">
+        <v>105.5</v>
+      </c>
+      <c r="GG36" t="n">
+        <v>105</v>
+      </c>
+      <c r="GH36" t="n">
+        <v>106.9</v>
+      </c>
+      <c r="GI36" t="n">
+        <v>105.9</v>
+      </c>
+      <c r="GJ36" t="n">
+        <v>101.3</v>
+      </c>
+      <c r="GK36" t="n">
+        <v>102.7</v>
       </c>
     </row>
     <row r="37">
@@ -18065,8 +18851,29 @@
       <c r="FN37" t="n">
         <v>103</v>
       </c>
+      <c r="FW37" t="n">
+        <v>100.75</v>
+      </c>
       <c r="FZ37" t="n">
         <v>112.9</v>
+      </c>
+      <c r="GE37" t="n">
+        <v>112.5</v>
+      </c>
+      <c r="GF37" t="n">
+        <v>105.25</v>
+      </c>
+      <c r="GG37" t="n">
+        <v>105</v>
+      </c>
+      <c r="GH37" t="n">
+        <v>106.9</v>
+      </c>
+      <c r="GJ37" t="n">
+        <v>101.45</v>
+      </c>
+      <c r="GK37" t="n">
+        <v>103.3</v>
       </c>
     </row>
     <row r="38">
@@ -18549,8 +19356,32 @@
       <c r="FP38" t="n">
         <v>100</v>
       </c>
+      <c r="FW38" t="n">
+        <v>100.5</v>
+      </c>
       <c r="FZ38" t="n">
         <v>112.9</v>
+      </c>
+      <c r="GE38" t="n">
+        <v>112.7</v>
+      </c>
+      <c r="GF38" t="n">
+        <v>106.5</v>
+      </c>
+      <c r="GG38" t="n">
+        <v>105</v>
+      </c>
+      <c r="GH38" t="n">
+        <v>106.95</v>
+      </c>
+      <c r="GI38" t="n">
+        <v>101.1</v>
+      </c>
+      <c r="GJ38" t="n">
+        <v>101.4</v>
+      </c>
+      <c r="GK38" t="n">
+        <v>102.55</v>
       </c>
     </row>
     <row r="39">
@@ -19042,8 +19873,35 @@
       <c r="FP39" t="n">
         <v>100.4</v>
       </c>
+      <c r="FW39" t="n">
+        <v>100.7</v>
+      </c>
       <c r="FZ39" t="n">
         <v>113.65</v>
+      </c>
+      <c r="GE39" t="n">
+        <v>112.8</v>
+      </c>
+      <c r="GF39" t="n">
+        <v>107</v>
+      </c>
+      <c r="GG39" t="n">
+        <v>105.2</v>
+      </c>
+      <c r="GH39" t="n">
+        <v>108.5</v>
+      </c>
+      <c r="GI39" t="n">
+        <v>103.2</v>
+      </c>
+      <c r="GJ39" t="n">
+        <v>101.4</v>
+      </c>
+      <c r="GK39" t="n">
+        <v>103.3</v>
+      </c>
+      <c r="GM39" t="n">
+        <v>104.05</v>
       </c>
     </row>
     <row r="40">
@@ -19529,8 +20387,35 @@
       <c r="FP40" t="n">
         <v>100.35</v>
       </c>
+      <c r="FW40" t="n">
+        <v>101.3</v>
+      </c>
       <c r="FZ40" t="n">
         <v>113.95</v>
+      </c>
+      <c r="GE40" t="n">
+        <v>115.15</v>
+      </c>
+      <c r="GF40" t="n">
+        <v>106.4</v>
+      </c>
+      <c r="GG40" t="n">
+        <v>106.4</v>
+      </c>
+      <c r="GH40" t="n">
+        <v>107.35</v>
+      </c>
+      <c r="GI40" t="n">
+        <v>103</v>
+      </c>
+      <c r="GJ40" t="n">
+        <v>102</v>
+      </c>
+      <c r="GK40" t="n">
+        <v>103</v>
+      </c>
+      <c r="GM40" t="n">
+        <v>103.7</v>
       </c>
     </row>
     <row r="41">
@@ -20022,6 +20907,27 @@
       <c r="FP41" t="n">
         <v>100.4</v>
       </c>
+      <c r="FW41" t="n">
+        <v>101.3</v>
+      </c>
+      <c r="GE41" t="n">
+        <v>113.65</v>
+      </c>
+      <c r="GF41" t="n">
+        <v>106.25</v>
+      </c>
+      <c r="GH41" t="n">
+        <v>107.35</v>
+      </c>
+      <c r="GI41" t="n">
+        <v>104.9</v>
+      </c>
+      <c r="GJ41" t="n">
+        <v>101.75</v>
+      </c>
+      <c r="GK41" t="n">
+        <v>103</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -20509,6 +21415,33 @@
       <c r="FP42" t="n">
         <v>100.05</v>
       </c>
+      <c r="FW42" t="n">
+        <v>101.25</v>
+      </c>
+      <c r="GE42" t="n">
+        <v>113.95</v>
+      </c>
+      <c r="GF42" t="n">
+        <v>105.85</v>
+      </c>
+      <c r="GG42" t="n">
+        <v>105.5</v>
+      </c>
+      <c r="GH42" t="n">
+        <v>107.35</v>
+      </c>
+      <c r="GI42" t="n">
+        <v>103</v>
+      </c>
+      <c r="GJ42" t="n">
+        <v>101.8</v>
+      </c>
+      <c r="GK42" t="n">
+        <v>102.75</v>
+      </c>
+      <c r="GM42" t="n">
+        <v>102.05</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -20996,8 +21929,32 @@
       <c r="FO43" t="n">
         <v>103.9</v>
       </c>
+      <c r="FW43" t="n">
+        <v>100.75</v>
+      </c>
       <c r="FZ43" t="n">
         <v>114.2</v>
+      </c>
+      <c r="GE43" t="n">
+        <v>113.7</v>
+      </c>
+      <c r="GF43" t="n">
+        <v>106.25</v>
+      </c>
+      <c r="GG43" t="n">
+        <v>106</v>
+      </c>
+      <c r="GH43" t="n">
+        <v>107.7</v>
+      </c>
+      <c r="GI43" t="n">
+        <v>103.6</v>
+      </c>
+      <c r="GJ43" t="n">
+        <v>101.5</v>
+      </c>
+      <c r="GK43" t="n">
+        <v>103</v>
       </c>
     </row>
     <row r="44">
@@ -21489,8 +22446,35 @@
       <c r="FP44" t="n">
         <v>100.05</v>
       </c>
+      <c r="FW44" t="n">
+        <v>101</v>
+      </c>
       <c r="FZ44" t="n">
         <v>114.4</v>
+      </c>
+      <c r="GE44" t="n">
+        <v>115.05</v>
+      </c>
+      <c r="GF44" t="n">
+        <v>106.5</v>
+      </c>
+      <c r="GG44" t="n">
+        <v>105.2</v>
+      </c>
+      <c r="GH44" t="n">
+        <v>107.4</v>
+      </c>
+      <c r="GI44" t="n">
+        <v>104.5</v>
+      </c>
+      <c r="GJ44" t="n">
+        <v>101.8</v>
+      </c>
+      <c r="GK44" t="n">
+        <v>103</v>
+      </c>
+      <c r="GM44" t="n">
+        <v>101</v>
       </c>
     </row>
     <row r="45">
@@ -21982,8 +22966,35 @@
       <c r="FP45" t="n">
         <v>100.55</v>
       </c>
+      <c r="FW45" t="n">
+        <v>101.3</v>
+      </c>
       <c r="FZ45" t="n">
         <v>114.45</v>
+      </c>
+      <c r="GE45" t="n">
+        <v>113.6</v>
+      </c>
+      <c r="GF45" t="n">
+        <v>107.7</v>
+      </c>
+      <c r="GG45" t="n">
+        <v>105</v>
+      </c>
+      <c r="GH45" t="n">
+        <v>107.6</v>
+      </c>
+      <c r="GI45" t="n">
+        <v>103</v>
+      </c>
+      <c r="GJ45" t="n">
+        <v>101.75</v>
+      </c>
+      <c r="GK45" t="n">
+        <v>103.3</v>
+      </c>
+      <c r="GM45" t="n">
+        <v>102.05</v>
       </c>
     </row>
     <row r="46">
@@ -22475,8 +23486,32 @@
       <c r="FP46" t="n">
         <v>100.75</v>
       </c>
+      <c r="FW46" t="n">
+        <v>101.75</v>
+      </c>
       <c r="FZ46" t="n">
         <v>111.45</v>
+      </c>
+      <c r="GE46" t="n">
+        <v>115</v>
+      </c>
+      <c r="GF46" t="n">
+        <v>106.45</v>
+      </c>
+      <c r="GG46" t="n">
+        <v>105.85</v>
+      </c>
+      <c r="GH46" t="n">
+        <v>107.5</v>
+      </c>
+      <c r="GI46" t="n">
+        <v>103.75</v>
+      </c>
+      <c r="GJ46" t="n">
+        <v>101.75</v>
+      </c>
+      <c r="GK46" t="n">
+        <v>103.3</v>
       </c>
     </row>
     <row r="47">
@@ -22971,8 +24006,32 @@
       <c r="FP47" t="n">
         <v>100.75</v>
       </c>
+      <c r="FW47" t="n">
+        <v>102</v>
+      </c>
       <c r="FZ47" t="n">
         <v>111.4</v>
+      </c>
+      <c r="GE47" t="n">
+        <v>113.95</v>
+      </c>
+      <c r="GF47" t="n">
+        <v>107</v>
+      </c>
+      <c r="GG47" t="n">
+        <v>105.25</v>
+      </c>
+      <c r="GH47" t="n">
+        <v>104.3</v>
+      </c>
+      <c r="GI47" t="n">
+        <v>103.3</v>
+      </c>
+      <c r="GJ47" t="n">
+        <v>101.85</v>
+      </c>
+      <c r="GK47" t="n">
+        <v>102.15</v>
       </c>
     </row>
     <row r="48">
@@ -23450,8 +24509,35 @@
       <c r="FN48" t="n">
         <v>103.75</v>
       </c>
+      <c r="FW48" t="n">
+        <v>101.2</v>
+      </c>
       <c r="FZ48" t="n">
         <v>110.95</v>
+      </c>
+      <c r="GE48" t="n">
+        <v>113.7</v>
+      </c>
+      <c r="GF48" t="n">
+        <v>106.3</v>
+      </c>
+      <c r="GG48" t="n">
+        <v>105.25</v>
+      </c>
+      <c r="GH48" t="n">
+        <v>104.7</v>
+      </c>
+      <c r="GI48" t="n">
+        <v>103.7</v>
+      </c>
+      <c r="GJ48" t="n">
+        <v>101.75</v>
+      </c>
+      <c r="GK48" t="n">
+        <v>102.85</v>
+      </c>
+      <c r="GM48" t="n">
+        <v>102</v>
       </c>
     </row>
     <row r="49">
@@ -23929,11 +25015,44 @@
       <c r="FP49" t="n">
         <v>100.6</v>
       </c>
+      <c r="FR49" t="n">
+        <v>147500</v>
+      </c>
+      <c r="FT49" t="n">
+        <v>100.65</v>
+      </c>
+      <c r="FW49" t="n">
+        <v>101.5</v>
+      </c>
       <c r="FZ49" t="n">
         <v>110.95</v>
       </c>
       <c r="GA49" t="n">
         <v>103</v>
+      </c>
+      <c r="GE49" t="n">
+        <v>113.95</v>
+      </c>
+      <c r="GF49" t="n">
+        <v>106.4</v>
+      </c>
+      <c r="GG49" t="n">
+        <v>105</v>
+      </c>
+      <c r="GH49" t="n">
+        <v>103.8</v>
+      </c>
+      <c r="GI49" t="n">
+        <v>103.35</v>
+      </c>
+      <c r="GJ49" t="n">
+        <v>101.25</v>
+      </c>
+      <c r="GK49" t="n">
+        <v>102.5</v>
+      </c>
+      <c r="GM49" t="n">
+        <v>101.5</v>
       </c>
     </row>
     <row r="50">
@@ -24446,6 +25565,33 @@
       <c r="GA50" t="n">
         <v>104</v>
       </c>
+      <c r="GE50" t="n">
+        <v>113.1</v>
+      </c>
+      <c r="GF50" t="n">
+        <v>106.7</v>
+      </c>
+      <c r="GG50" t="n">
+        <v>105.5</v>
+      </c>
+      <c r="GH50" t="n">
+        <v>104.2</v>
+      </c>
+      <c r="GI50" t="n">
+        <v>104</v>
+      </c>
+      <c r="GJ50" t="n">
+        <v>101.35</v>
+      </c>
+      <c r="GK50" t="n">
+        <v>101.95</v>
+      </c>
+      <c r="GL50" t="n">
+        <v>33</v>
+      </c>
+      <c r="GM50" t="n">
+        <v>101</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -24948,6 +26094,30 @@
       <c r="GA51" t="n">
         <v>103.1</v>
       </c>
+      <c r="GE51" t="n">
+        <v>113.85</v>
+      </c>
+      <c r="GF51" t="n">
+        <v>106.15</v>
+      </c>
+      <c r="GG51" t="n">
+        <v>105.5</v>
+      </c>
+      <c r="GH51" t="n">
+        <v>103.85</v>
+      </c>
+      <c r="GI51" t="n">
+        <v>104</v>
+      </c>
+      <c r="GJ51" t="n">
+        <v>101</v>
+      </c>
+      <c r="GK51" t="n">
+        <v>102.7</v>
+      </c>
+      <c r="GL51" t="n">
+        <v>29.8</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -25450,6 +26620,33 @@
       <c r="GA52" t="n">
         <v>104</v>
       </c>
+      <c r="GE52" t="n">
+        <v>113.9</v>
+      </c>
+      <c r="GF52" t="n">
+        <v>106.75</v>
+      </c>
+      <c r="GG52" t="n">
+        <v>105.8</v>
+      </c>
+      <c r="GH52" t="n">
+        <v>103.9</v>
+      </c>
+      <c r="GI52" t="n">
+        <v>103.25</v>
+      </c>
+      <c r="GJ52" t="n">
+        <v>101</v>
+      </c>
+      <c r="GK52" t="n">
+        <v>102.8</v>
+      </c>
+      <c r="GL52" t="n">
+        <v>29.006</v>
+      </c>
+      <c r="GM52" t="n">
+        <v>101.95</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="4" t="n">
@@ -25953,6 +27150,36 @@
       <c r="GA53" t="n">
         <v>104.05</v>
       </c>
+      <c r="GB53" t="n">
+        <v>100.05</v>
+      </c>
+      <c r="GE53" t="n">
+        <v>113.75</v>
+      </c>
+      <c r="GF53" t="n">
+        <v>106.5</v>
+      </c>
+      <c r="GG53" t="n">
+        <v>105.6</v>
+      </c>
+      <c r="GH53" t="n">
+        <v>104.45</v>
+      </c>
+      <c r="GI53" t="n">
+        <v>103.25</v>
+      </c>
+      <c r="GJ53" t="n">
+        <v>101.5</v>
+      </c>
+      <c r="GK53" t="n">
+        <v>103.25</v>
+      </c>
+      <c r="GL53" t="n">
+        <v>30.712</v>
+      </c>
+      <c r="GM53" t="n">
+        <v>99.99999999999999</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="3" t="n">
@@ -26455,6 +27682,36 @@
       </c>
       <c r="GA54" t="n">
         <v>104.25</v>
+      </c>
+      <c r="GB54" t="n">
+        <v>101.35</v>
+      </c>
+      <c r="GE54" t="n">
+        <v>113.95</v>
+      </c>
+      <c r="GF54" t="n">
+        <v>106.1</v>
+      </c>
+      <c r="GG54" t="n">
+        <v>105.8</v>
+      </c>
+      <c r="GH54" t="n">
+        <v>104.4</v>
+      </c>
+      <c r="GI54" t="n">
+        <v>103.05</v>
+      </c>
+      <c r="GJ54" t="n">
+        <v>100.6</v>
+      </c>
+      <c r="GK54" t="n">
+        <v>102.7</v>
+      </c>
+      <c r="GL54" t="n">
+        <v>34</v>
+      </c>
+      <c r="GM54" t="n">
+        <v>102</v>
       </c>
     </row>
     <row r="55">
@@ -26931,6 +28188,9 @@
       <c r="FQ55" t="n">
         <v>100.69</v>
       </c>
+      <c r="FR55" t="n">
+        <v>147950</v>
+      </c>
       <c r="FS55" t="n">
         <v>137100</v>
       </c>
@@ -26957,6 +28217,30 @@
       </c>
       <c r="GB55" t="n">
         <v>101</v>
+      </c>
+      <c r="GE55" t="n">
+        <v>113.85</v>
+      </c>
+      <c r="GF55" t="n">
+        <v>106.35</v>
+      </c>
+      <c r="GG55" t="n">
+        <v>105.45</v>
+      </c>
+      <c r="GH55" t="n">
+        <v>104</v>
+      </c>
+      <c r="GI55" t="n">
+        <v>103.7</v>
+      </c>
+      <c r="GJ55" t="n">
+        <v>101.65</v>
+      </c>
+      <c r="GK55" t="n">
+        <v>103</v>
+      </c>
+      <c r="GM55" t="n">
+        <v>100.55</v>
       </c>
     </row>
     <row r="56">
@@ -27439,6 +28723,9 @@
       <c r="FQ56" t="n">
         <v>100.77</v>
       </c>
+      <c r="FR56" t="n">
+        <v>148000</v>
+      </c>
       <c r="FS56" t="n">
         <v>136900</v>
       </c>
@@ -27465,6 +28752,33 @@
       </c>
       <c r="GB56" t="n">
         <v>100.85</v>
+      </c>
+      <c r="GE56" t="n">
+        <v>114</v>
+      </c>
+      <c r="GF56" t="n">
+        <v>106.7</v>
+      </c>
+      <c r="GG56" t="n">
+        <v>105.1</v>
+      </c>
+      <c r="GH56" t="n">
+        <v>104</v>
+      </c>
+      <c r="GI56" t="n">
+        <v>103.6</v>
+      </c>
+      <c r="GJ56" t="n">
+        <v>101.6</v>
+      </c>
+      <c r="GK56" t="n">
+        <v>103</v>
+      </c>
+      <c r="GL56" t="n">
+        <v>31.5</v>
+      </c>
+      <c r="GM56" t="n">
+        <v>102.1</v>
       </c>
     </row>
     <row r="57">
@@ -27944,6 +29258,9 @@
       <c r="FQ57" t="n">
         <v>100.9</v>
       </c>
+      <c r="FR57" t="n">
+        <v>148000</v>
+      </c>
       <c r="FS57" t="n">
         <v>136890</v>
       </c>
@@ -27953,6 +29270,9 @@
       <c r="FV57" t="n">
         <v>100.3</v>
       </c>
+      <c r="FW57" t="n">
+        <v>102.1</v>
+      </c>
       <c r="FX57" t="n">
         <v>103.65</v>
       </c>
@@ -27967,6 +29287,30 @@
       </c>
       <c r="GB57" t="n">
         <v>100.85</v>
+      </c>
+      <c r="GE57" t="n">
+        <v>114.45</v>
+      </c>
+      <c r="GF57" t="n">
+        <v>106.4</v>
+      </c>
+      <c r="GG57" t="n">
+        <v>104.85</v>
+      </c>
+      <c r="GH57" t="n">
+        <v>104.05</v>
+      </c>
+      <c r="GI57" t="n">
+        <v>104.9</v>
+      </c>
+      <c r="GJ57" t="n">
+        <v>101.1</v>
+      </c>
+      <c r="GK57" t="n">
+        <v>103.3</v>
+      </c>
+      <c r="GM57" t="n">
+        <v>102</v>
       </c>
     </row>
     <row r="58">
@@ -28443,6 +29787,9 @@
       <c r="FQ58" t="n">
         <v>100.999</v>
       </c>
+      <c r="FR58" t="n">
+        <v>149000</v>
+      </c>
       <c r="FS58" t="n">
         <v>136690</v>
       </c>
@@ -28466,6 +29813,33 @@
       </c>
       <c r="GB58" t="n">
         <v>100.45</v>
+      </c>
+      <c r="GE58" t="n">
+        <v>114.35</v>
+      </c>
+      <c r="GF58" t="n">
+        <v>106.3</v>
+      </c>
+      <c r="GG58" t="n">
+        <v>104.8</v>
+      </c>
+      <c r="GH58" t="n">
+        <v>104.05</v>
+      </c>
+      <c r="GI58" t="n">
+        <v>104.9</v>
+      </c>
+      <c r="GJ58" t="n">
+        <v>100.8</v>
+      </c>
+      <c r="GK58" t="n">
+        <v>103.3</v>
+      </c>
+      <c r="GL58" t="n">
+        <v>32</v>
+      </c>
+      <c r="GM58" t="n">
+        <v>100</v>
       </c>
     </row>
     <row r="59">
@@ -28939,6 +30313,9 @@
       <c r="FQ59" t="n">
         <v>101.18</v>
       </c>
+      <c r="FR59" t="n">
+        <v>149000</v>
+      </c>
       <c r="FS59" t="n">
         <v>136740</v>
       </c>
@@ -28948,6 +30325,9 @@
       <c r="FV59" t="n">
         <v>99.95</v>
       </c>
+      <c r="FW59" t="n">
+        <v>102.75</v>
+      </c>
       <c r="FX59" t="n">
         <v>103.95</v>
       </c>
@@ -28962,6 +30342,39 @@
       </c>
       <c r="GB59" t="n">
         <v>101</v>
+      </c>
+      <c r="GC59" t="n">
+        <v>98.25</v>
+      </c>
+      <c r="GD59" t="n">
+        <v>147690</v>
+      </c>
+      <c r="GE59" t="n">
+        <v>114.25</v>
+      </c>
+      <c r="GF59" t="n">
+        <v>106.25</v>
+      </c>
+      <c r="GG59" t="n">
+        <v>104.3</v>
+      </c>
+      <c r="GH59" t="n">
+        <v>104.2</v>
+      </c>
+      <c r="GI59" t="n">
+        <v>102.55</v>
+      </c>
+      <c r="GJ59" t="n">
+        <v>101.65</v>
+      </c>
+      <c r="GK59" t="n">
+        <v>103</v>
+      </c>
+      <c r="GL59" t="n">
+        <v>31</v>
+      </c>
+      <c r="GM59" t="n">
+        <v>100.15</v>
       </c>
     </row>
     <row r="60">
@@ -29477,6 +30890,33 @@
       <c r="GD60" t="n">
         <v>147920</v>
       </c>
+      <c r="GE60" t="n">
+        <v>113.9</v>
+      </c>
+      <c r="GF60" t="n">
+        <v>106</v>
+      </c>
+      <c r="GG60" t="n">
+        <v>104.5</v>
+      </c>
+      <c r="GH60" t="n">
+        <v>104.3</v>
+      </c>
+      <c r="GI60" t="n">
+        <v>104</v>
+      </c>
+      <c r="GJ60" t="n">
+        <v>101.2</v>
+      </c>
+      <c r="GK60" t="n">
+        <v>102.9</v>
+      </c>
+      <c r="GL60" t="n">
+        <v>30.204</v>
+      </c>
+      <c r="GM60" t="n">
+        <v>100.15</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">

</xml_diff>

<commit_message>
Completar ruedas: convertir por canje los CCL sin cotizar, y recuperar el 25/08
completar_ruedas sólo miraba plan[f], que sale de faltantes(): ese filtro exige que el
ticker haya cotizado en la rueda sana anterior, justamente lo que los papeles que nunca
operan en CCL no cumplen. El hueco de ellos es estructural, no una rueda rota, así que
por ese camino no entraban nunca. Ahora el paso de canje barre todo el universo en CCL:
el precio que se busca ahí es el MEP, y ese sí existe.

Se recupera la rueda del 25/08, que el job dejó con 18 CCL vacíos por el fallo de BYMA:
17 completados (ERM33 no tuvo precio en ninguna de las dos puntas). Variaciones contra
el 24/08 dentro de +-3%, sin el salto de ~3,6% que delataría una punta cruzada.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/historicos.xlsx
+++ b/historicos.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="760" windowWidth="29400" windowHeight="16980" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Historicos" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Historicos" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -33262,6 +33262,9 @@
       <c r="BO65" t="n">
         <v>109.5</v>
       </c>
+      <c r="BP65" t="n">
+        <v>104.0928</v>
+      </c>
       <c r="BQ65" t="n">
         <v>150650</v>
       </c>
@@ -33310,15 +33313,30 @@
       <c r="CG65" t="n">
         <v>103.35</v>
       </c>
+      <c r="CH65" t="n">
+        <v>46.2742</v>
+      </c>
+      <c r="CI65" t="n">
+        <v>61.7823</v>
+      </c>
+      <c r="CJ65" t="n">
+        <v>106.3055</v>
+      </c>
       <c r="CL65" t="n">
         <v>101.45</v>
       </c>
+      <c r="CM65" t="n">
+        <v>98.994</v>
+      </c>
       <c r="CN65" t="n">
         <v>100.9</v>
       </c>
       <c r="CO65" t="n">
         <v>74.3</v>
       </c>
+      <c r="CP65" t="n">
+        <v>75.0873</v>
+      </c>
       <c r="CQ65" t="n">
         <v>105.95</v>
       </c>
@@ -33337,6 +33355,9 @@
       <c r="CV65" t="n">
         <v>80.69</v>
       </c>
+      <c r="CW65" t="n">
+        <v>49.3142</v>
+      </c>
       <c r="CX65" t="n">
         <v>108.9</v>
       </c>
@@ -33346,6 +33367,12 @@
       <c r="CZ65" t="n">
         <v>99.90000000000001</v>
       </c>
+      <c r="DA65" t="n">
+        <v>108.1334</v>
+      </c>
+      <c r="DB65" t="n">
+        <v>105.0548</v>
+      </c>
       <c r="DC65" t="n">
         <v>103.2</v>
       </c>
@@ -33370,9 +33397,18 @@
       <c r="DJ65" t="n">
         <v>104.75</v>
       </c>
+      <c r="DK65" t="n">
+        <v>107.027</v>
+      </c>
+      <c r="DL65" t="n">
+        <v>105.0548</v>
+      </c>
       <c r="DM65" t="n">
         <v>107.85</v>
       </c>
+      <c r="DN65" t="n">
+        <v>104.5738</v>
+      </c>
       <c r="DO65" t="n">
         <v>105.9</v>
       </c>
@@ -33544,12 +33580,21 @@
       <c r="FV65" t="n">
         <v>99.30000000000001</v>
       </c>
+      <c r="FW65" t="n">
+        <v>98.5611</v>
+      </c>
+      <c r="FX65" t="n">
+        <v>99.5712</v>
+      </c>
       <c r="FY65" t="n">
         <v>25.571</v>
       </c>
       <c r="FZ65" t="n">
         <v>107.9</v>
       </c>
+      <c r="GA65" t="n">
+        <v>99.956</v>
+      </c>
       <c r="GB65" t="n">
         <v>100.2</v>
       </c>
@@ -33559,6 +33604,9 @@
       <c r="GD65" t="n">
         <v>149450</v>
       </c>
+      <c r="GE65" t="n">
+        <v>109.1916</v>
+      </c>
       <c r="GF65" t="n">
         <v>106.05</v>
       </c>
@@ -33576,6 +33624,9 @@
       </c>
       <c r="GK65" t="n">
         <v>103</v>
+      </c>
+      <c r="GL65" t="n">
+        <v>28.8131</v>
       </c>
       <c r="GM65" t="n">
         <v>101</v>

</xml_diff>

<commit_message>
Rellenar historia de instrumentos nuevos 2026-09-03
</commit_message>
<xml_diff>
--- a/historicos.xlsx
+++ b/historicos.xlsx
@@ -1898,6 +1898,9 @@
       <c r="GS2" t="n">
         <v>37280</v>
       </c>
+      <c r="GZ2" t="n">
+        <v>102</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -2370,6 +2373,15 @@
       <c r="GS3" t="n">
         <v>42060</v>
       </c>
+      <c r="GX3" t="n">
+        <v>104</v>
+      </c>
+      <c r="GY3" t="n">
+        <v>99</v>
+      </c>
+      <c r="GZ3" t="n">
+        <v>104.75</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -2845,6 +2857,15 @@
       <c r="GS4" t="n">
         <v>41985</v>
       </c>
+      <c r="GX4" t="n">
+        <v>103.5</v>
+      </c>
+      <c r="GY4" t="n">
+        <v>100</v>
+      </c>
+      <c r="GZ4" t="n">
+        <v>103.85</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -3323,6 +3344,15 @@
       <c r="GS5" t="n">
         <v>41900</v>
       </c>
+      <c r="GX5" t="n">
+        <v>104.3</v>
+      </c>
+      <c r="GY5" t="n">
+        <v>97.01000000000001</v>
+      </c>
+      <c r="GZ5" t="n">
+        <v>104.1</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -3810,6 +3840,15 @@
       <c r="GS6" t="n">
         <v>41865</v>
       </c>
+      <c r="GX6" t="n">
+        <v>104.3</v>
+      </c>
+      <c r="GY6" t="n">
+        <v>100.5</v>
+      </c>
+      <c r="GZ6" t="n">
+        <v>104.05</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -4309,6 +4348,15 @@
       <c r="GS7" t="n">
         <v>41800</v>
       </c>
+      <c r="GX7" t="n">
+        <v>104.15</v>
+      </c>
+      <c r="GY7" t="n">
+        <v>100.5</v>
+      </c>
+      <c r="GZ7" t="n">
+        <v>104.15</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -4802,6 +4850,15 @@
       <c r="GS8" t="n">
         <v>42150</v>
       </c>
+      <c r="GX8" t="n">
+        <v>103.95</v>
+      </c>
+      <c r="GY8" t="n">
+        <v>100.5</v>
+      </c>
+      <c r="GZ8" t="n">
+        <v>104.25</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -5301,6 +5358,12 @@
       <c r="GS9" t="n">
         <v>42900</v>
       </c>
+      <c r="GX9" t="n">
+        <v>103.55</v>
+      </c>
+      <c r="GZ9" t="n">
+        <v>104.45</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -5803,6 +5866,15 @@
       <c r="GS10" t="n">
         <v>42795</v>
       </c>
+      <c r="GX10" t="n">
+        <v>103.35</v>
+      </c>
+      <c r="GY10" t="n">
+        <v>98.00000000000001</v>
+      </c>
+      <c r="GZ10" t="n">
+        <v>104.8</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -6293,6 +6365,12 @@
       <c r="GS11" t="n">
         <v>43000</v>
       </c>
+      <c r="GX11" t="n">
+        <v>104.3</v>
+      </c>
+      <c r="GZ11" t="n">
+        <v>104.25</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -6780,6 +6858,12 @@
       <c r="GS12" t="n">
         <v>42705</v>
       </c>
+      <c r="GX12" t="n">
+        <v>103.8</v>
+      </c>
+      <c r="GZ12" t="n">
+        <v>104.2</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -7282,6 +7366,12 @@
       <c r="GS13" t="n">
         <v>43100</v>
       </c>
+      <c r="GX13" t="n">
+        <v>104.4</v>
+      </c>
+      <c r="GZ13" t="n">
+        <v>104.35</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -7784,6 +7874,12 @@
       <c r="GS14" t="n">
         <v>43550</v>
       </c>
+      <c r="GX14" t="n">
+        <v>103.7</v>
+      </c>
+      <c r="GZ14" t="n">
+        <v>104.35</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -8280,6 +8376,12 @@
       <c r="GS15" t="n">
         <v>44130</v>
       </c>
+      <c r="GX15" t="n">
+        <v>104</v>
+      </c>
+      <c r="GZ15" t="n">
+        <v>104.5</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -8794,6 +8896,12 @@
       <c r="GS16" t="n">
         <v>43700</v>
       </c>
+      <c r="GX16" t="n">
+        <v>104.4</v>
+      </c>
+      <c r="GZ16" t="n">
+        <v>104.15</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -9305,6 +9413,12 @@
       <c r="GS17" t="n">
         <v>43650</v>
       </c>
+      <c r="GX17" t="n">
+        <v>105.4</v>
+      </c>
+      <c r="GZ17" t="n">
+        <v>104.35</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -9813,6 +9927,12 @@
       <c r="GS18" t="n">
         <v>44390</v>
       </c>
+      <c r="GX18" t="n">
+        <v>104.95</v>
+      </c>
+      <c r="GZ18" t="n">
+        <v>105.35</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -10327,6 +10447,12 @@
       <c r="GS19" t="n">
         <v>44970</v>
       </c>
+      <c r="GX19" t="n">
+        <v>105.05</v>
+      </c>
+      <c r="GZ19" t="n">
+        <v>104.35</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -10838,6 +10964,12 @@
       <c r="GS20" t="n">
         <v>45600</v>
       </c>
+      <c r="GX20" t="n">
+        <v>104.95</v>
+      </c>
+      <c r="GZ20" t="n">
+        <v>104.45</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -11349,6 +11481,15 @@
       <c r="GS21" t="n">
         <v>45970</v>
       </c>
+      <c r="GX21" t="n">
+        <v>104.15</v>
+      </c>
+      <c r="GY21" t="n">
+        <v>101</v>
+      </c>
+      <c r="GZ21" t="n">
+        <v>104.45</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -11869,6 +12010,18 @@
       <c r="GS22" t="n">
         <v>46000</v>
       </c>
+      <c r="GW22" t="n">
+        <v>101</v>
+      </c>
+      <c r="GX22" t="n">
+        <v>104.15</v>
+      </c>
+      <c r="GY22" t="n">
+        <v>97.56</v>
+      </c>
+      <c r="GZ22" t="n">
+        <v>104.3</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -12386,6 +12539,15 @@
       <c r="GS23" t="n">
         <v>46160</v>
       </c>
+      <c r="GW23" t="n">
+        <v>101.05</v>
+      </c>
+      <c r="GX23" t="n">
+        <v>104.5</v>
+      </c>
+      <c r="GZ23" t="n">
+        <v>104.1</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -12903,6 +13065,18 @@
       <c r="GS24" t="n">
         <v>45935</v>
       </c>
+      <c r="GW24" t="n">
+        <v>101.1</v>
+      </c>
+      <c r="GX24" t="n">
+        <v>105.1</v>
+      </c>
+      <c r="GY24" t="n">
+        <v>101.4</v>
+      </c>
+      <c r="GZ24" t="n">
+        <v>103.5</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -13417,6 +13591,18 @@
       <c r="GS25" t="n">
         <v>45900</v>
       </c>
+      <c r="GW25" t="n">
+        <v>100.4</v>
+      </c>
+      <c r="GX25" t="n">
+        <v>105.55</v>
+      </c>
+      <c r="GY25" t="n">
+        <v>101.7</v>
+      </c>
+      <c r="GZ25" t="n">
+        <v>104.3</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -13925,6 +14111,15 @@
       <c r="GS26" t="n">
         <v>45945</v>
       </c>
+      <c r="GW26" t="n">
+        <v>101.7</v>
+      </c>
+      <c r="GX26" t="n">
+        <v>105.5</v>
+      </c>
+      <c r="GZ26" t="n">
+        <v>105.2</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -14436,6 +14631,18 @@
       <c r="GS27" t="n">
         <v>46400</v>
       </c>
+      <c r="GW27" t="n">
+        <v>101</v>
+      </c>
+      <c r="GX27" t="n">
+        <v>105.4</v>
+      </c>
+      <c r="GY27" t="n">
+        <v>98.90000000000001</v>
+      </c>
+      <c r="GZ27" t="n">
+        <v>104.95</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -14950,6 +15157,18 @@
       <c r="GS28" t="n">
         <v>46750</v>
       </c>
+      <c r="GW28" t="n">
+        <v>101.1</v>
+      </c>
+      <c r="GX28" t="n">
+        <v>105.1</v>
+      </c>
+      <c r="GY28" t="n">
+        <v>100.5</v>
+      </c>
+      <c r="GZ28" t="n">
+        <v>104.6</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -15473,6 +15692,18 @@
       <c r="GS29" t="n">
         <v>47340</v>
       </c>
+      <c r="GW29" t="n">
+        <v>100.95</v>
+      </c>
+      <c r="GX29" t="n">
+        <v>105</v>
+      </c>
+      <c r="GY29" t="n">
+        <v>102</v>
+      </c>
+      <c r="GZ29" t="n">
+        <v>104.15</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -15996,6 +16227,15 @@
       <c r="GS30" t="n">
         <v>46980</v>
       </c>
+      <c r="GW30" t="n">
+        <v>101.1</v>
+      </c>
+      <c r="GX30" t="n">
+        <v>105</v>
+      </c>
+      <c r="GZ30" t="n">
+        <v>104.65</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -16525,6 +16765,18 @@
       <c r="GS31" t="n">
         <v>47000</v>
       </c>
+      <c r="GW31" t="n">
+        <v>100.75</v>
+      </c>
+      <c r="GX31" t="n">
+        <v>105.45</v>
+      </c>
+      <c r="GY31" t="n">
+        <v>103</v>
+      </c>
+      <c r="GZ31" t="n">
+        <v>104.75</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -17045,6 +17297,18 @@
       <c r="GS32" t="n">
         <v>46995</v>
       </c>
+      <c r="GW32" t="n">
+        <v>100.8</v>
+      </c>
+      <c r="GX32" t="n">
+        <v>106.5</v>
+      </c>
+      <c r="GY32" t="n">
+        <v>98.3</v>
+      </c>
+      <c r="GZ32" t="n">
+        <v>104.8</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -17574,6 +17838,15 @@
       <c r="GS33" t="n">
         <v>47070</v>
       </c>
+      <c r="GW33" t="n">
+        <v>101.8</v>
+      </c>
+      <c r="GX33" t="n">
+        <v>105.75</v>
+      </c>
+      <c r="GZ33" t="n">
+        <v>104.6</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -18034,6 +18307,18 @@
       <c r="GS34" t="n">
         <v>47200</v>
       </c>
+      <c r="GW34" t="n">
+        <v>102</v>
+      </c>
+      <c r="GX34" t="n">
+        <v>107.1</v>
+      </c>
+      <c r="GY34" t="n">
+        <v>103</v>
+      </c>
+      <c r="GZ34" t="n">
+        <v>104.35</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -18563,6 +18848,18 @@
       <c r="GS35" t="n">
         <v>46780</v>
       </c>
+      <c r="GW35" t="n">
+        <v>101.8</v>
+      </c>
+      <c r="GX35" t="n">
+        <v>105.95</v>
+      </c>
+      <c r="GY35" t="n">
+        <v>103</v>
+      </c>
+      <c r="GZ35" t="n">
+        <v>104.45</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -19092,6 +19389,15 @@
       <c r="GS36" t="n">
         <v>46370</v>
       </c>
+      <c r="GW36" t="n">
+        <v>102</v>
+      </c>
+      <c r="GX36" t="n">
+        <v>106.3</v>
+      </c>
+      <c r="GZ36" t="n">
+        <v>104.75</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -19615,6 +19921,18 @@
       <c r="GS37" t="n">
         <v>46060</v>
       </c>
+      <c r="GW37" t="n">
+        <v>101.6</v>
+      </c>
+      <c r="GX37" t="n">
+        <v>106.9</v>
+      </c>
+      <c r="GY37" t="n">
+        <v>104.2</v>
+      </c>
+      <c r="GZ37" t="n">
+        <v>104.6</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -20141,6 +20459,18 @@
       <c r="GS38" t="n">
         <v>46090</v>
       </c>
+      <c r="GW38" t="n">
+        <v>101.4</v>
+      </c>
+      <c r="GX38" t="n">
+        <v>106.85</v>
+      </c>
+      <c r="GY38" t="n">
+        <v>103.5</v>
+      </c>
+      <c r="GZ38" t="n">
+        <v>104.8</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -20682,6 +21012,18 @@
       <c r="GS39" t="n">
         <v>46100</v>
       </c>
+      <c r="GW39" t="n">
+        <v>101.5</v>
+      </c>
+      <c r="GX39" t="n">
+        <v>106.5</v>
+      </c>
+      <c r="GY39" t="n">
+        <v>102.8</v>
+      </c>
+      <c r="GZ39" t="n">
+        <v>105.4</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -21214,6 +21556,18 @@
       <c r="GS40" t="n">
         <v>46880</v>
       </c>
+      <c r="GW40" t="n">
+        <v>101</v>
+      </c>
+      <c r="GX40" t="n">
+        <v>106.85</v>
+      </c>
+      <c r="GY40" t="n">
+        <v>103</v>
+      </c>
+      <c r="GZ40" t="n">
+        <v>105</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -21746,6 +22100,18 @@
       <c r="GS41" t="n">
         <v>47100</v>
       </c>
+      <c r="GW41" t="n">
+        <v>101.5</v>
+      </c>
+      <c r="GX41" t="n">
+        <v>106.75</v>
+      </c>
+      <c r="GY41" t="n">
+        <v>103</v>
+      </c>
+      <c r="GZ41" t="n">
+        <v>104.85</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -22281,6 +22647,15 @@
       <c r="GS42" t="n">
         <v>47010</v>
       </c>
+      <c r="GW42" t="n">
+        <v>101.05</v>
+      </c>
+      <c r="GX42" t="n">
+        <v>103.2</v>
+      </c>
+      <c r="GZ42" t="n">
+        <v>104.95</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -22813,6 +23188,15 @@
       <c r="GS43" t="n">
         <v>47150</v>
       </c>
+      <c r="GW43" t="n">
+        <v>101.4</v>
+      </c>
+      <c r="GX43" t="n">
+        <v>103.2</v>
+      </c>
+      <c r="GZ43" t="n">
+        <v>104.9</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -23354,6 +23738,18 @@
       <c r="GS44" t="n">
         <v>47150</v>
       </c>
+      <c r="GW44" t="n">
+        <v>101.3</v>
+      </c>
+      <c r="GX44" t="n">
+        <v>102.7</v>
+      </c>
+      <c r="GY44" t="n">
+        <v>102</v>
+      </c>
+      <c r="GZ44" t="n">
+        <v>105.4</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -23895,6 +24291,18 @@
       <c r="GS45" t="n">
         <v>47140</v>
       </c>
+      <c r="GW45" t="n">
+        <v>101.3</v>
+      </c>
+      <c r="GX45" t="n">
+        <v>103</v>
+      </c>
+      <c r="GY45" t="n">
+        <v>103</v>
+      </c>
+      <c r="GZ45" t="n">
+        <v>104.9</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -24433,6 +24841,18 @@
       <c r="GS46" t="n">
         <v>47250</v>
       </c>
+      <c r="GW46" t="n">
+        <v>101.55</v>
+      </c>
+      <c r="GX46" t="n">
+        <v>103</v>
+      </c>
+      <c r="GY46" t="n">
+        <v>102.9</v>
+      </c>
+      <c r="GZ46" t="n">
+        <v>104.95</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -24971,6 +25391,18 @@
       <c r="GS47" t="n">
         <v>46800</v>
       </c>
+      <c r="GW47" t="n">
+        <v>101.55</v>
+      </c>
+      <c r="GX47" t="n">
+        <v>103.25</v>
+      </c>
+      <c r="GY47" t="n">
+        <v>102.9</v>
+      </c>
+      <c r="GZ47" t="n">
+        <v>104.95</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="3" t="n">
@@ -25498,6 +25930,18 @@
       <c r="GS48" t="n">
         <v>46195</v>
       </c>
+      <c r="GW48" t="n">
+        <v>101.3</v>
+      </c>
+      <c r="GX48" t="n">
+        <v>103.2</v>
+      </c>
+      <c r="GY48" t="n">
+        <v>102.9</v>
+      </c>
+      <c r="GZ48" t="n">
+        <v>104.6</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="3" t="n">
@@ -26036,6 +26480,18 @@
       </c>
       <c r="GS49" t="n">
         <v>46200</v>
+      </c>
+      <c r="GW49" t="n">
+        <v>101.4</v>
+      </c>
+      <c r="GX49" t="n">
+        <v>103.4</v>
+      </c>
+      <c r="GY49" t="n">
+        <v>102.95</v>
+      </c>
+      <c r="GZ49" t="n">
+        <v>104.95</v>
       </c>
     </row>
     <row r="50">
@@ -26593,6 +27049,18 @@
       <c r="GS50" t="n">
         <v>46220</v>
       </c>
+      <c r="GW50" t="n">
+        <v>101.5</v>
+      </c>
+      <c r="GX50" t="n">
+        <v>103</v>
+      </c>
+      <c r="GY50" t="n">
+        <v>102.95</v>
+      </c>
+      <c r="GZ50" t="n">
+        <v>104.95</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -27140,6 +27608,18 @@
       <c r="GS51" t="n">
         <v>45995</v>
       </c>
+      <c r="GW51" t="n">
+        <v>101.4</v>
+      </c>
+      <c r="GX51" t="n">
+        <v>102.7</v>
+      </c>
+      <c r="GY51" t="n">
+        <v>103.25</v>
+      </c>
+      <c r="GZ51" t="n">
+        <v>105</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -27687,6 +28167,18 @@
       <c r="GS52" t="n">
         <v>45840</v>
       </c>
+      <c r="GW52" t="n">
+        <v>101.65</v>
+      </c>
+      <c r="GX52" t="n">
+        <v>103.15</v>
+      </c>
+      <c r="GY52" t="n">
+        <v>103</v>
+      </c>
+      <c r="GZ52" t="n">
+        <v>104.85</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="4" t="n">
@@ -28241,6 +28733,18 @@
       <c r="GS53" t="n">
         <v>44600</v>
       </c>
+      <c r="GW53" t="n">
+        <v>102</v>
+      </c>
+      <c r="GX53" t="n">
+        <v>102.9</v>
+      </c>
+      <c r="GY53" t="n">
+        <v>103.2</v>
+      </c>
+      <c r="GZ53" t="n">
+        <v>105</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="3" t="n">
@@ -28791,6 +29295,18 @@
       </c>
       <c r="GS54" t="n">
         <v>44110</v>
+      </c>
+      <c r="GW54" t="n">
+        <v>102.4</v>
+      </c>
+      <c r="GX54" t="n">
+        <v>102.8</v>
+      </c>
+      <c r="GY54" t="n">
+        <v>103.25</v>
+      </c>
+      <c r="GZ54" t="n">
+        <v>105</v>
       </c>
     </row>
     <row r="55">
@@ -29345,6 +29861,18 @@
       <c r="GS55" t="n">
         <v>43900</v>
       </c>
+      <c r="GW55" t="n">
+        <v>102.35</v>
+      </c>
+      <c r="GX55" t="n">
+        <v>103.1</v>
+      </c>
+      <c r="GY55" t="n">
+        <v>102.4</v>
+      </c>
+      <c r="GZ55" t="n">
+        <v>105.45</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -29901,6 +30429,18 @@
       <c r="GS56" t="n">
         <v>44200</v>
       </c>
+      <c r="GW56" t="n">
+        <v>101.75</v>
+      </c>
+      <c r="GX56" t="n">
+        <v>102.75</v>
+      </c>
+      <c r="GY56" t="n">
+        <v>103.25</v>
+      </c>
+      <c r="GZ56" t="n">
+        <v>105</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -30451,6 +30991,18 @@
       <c r="GS57" t="n">
         <v>43650</v>
       </c>
+      <c r="GW57" t="n">
+        <v>102</v>
+      </c>
+      <c r="GX57" t="n">
+        <v>102.8</v>
+      </c>
+      <c r="GY57" t="n">
+        <v>103.25</v>
+      </c>
+      <c r="GZ57" t="n">
+        <v>105.1</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -30998,6 +31550,18 @@
       <c r="GS58" t="n">
         <v>43750</v>
       </c>
+      <c r="GW58" t="n">
+        <v>101.95</v>
+      </c>
+      <c r="GX58" t="n">
+        <v>103.1</v>
+      </c>
+      <c r="GY58" t="n">
+        <v>103.25</v>
+      </c>
+      <c r="GZ58" t="n">
+        <v>105</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -31551,6 +32115,18 @@
       <c r="GS59" t="n">
         <v>43600</v>
       </c>
+      <c r="GW59" t="n">
+        <v>101.5</v>
+      </c>
+      <c r="GX59" t="n">
+        <v>102.8</v>
+      </c>
+      <c r="GY59" t="n">
+        <v>103</v>
+      </c>
+      <c r="GZ59" t="n">
+        <v>105.2</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -32110,6 +32686,18 @@
       <c r="GS60" t="n">
         <v>43000</v>
       </c>
+      <c r="GW60" t="n">
+        <v>101.6</v>
+      </c>
+      <c r="GX60" t="n">
+        <v>103.1</v>
+      </c>
+      <c r="GY60" t="n">
+        <v>102.3</v>
+      </c>
+      <c r="GZ60" t="n">
+        <v>105.5</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -32666,6 +33254,18 @@
       <c r="GS61" t="n">
         <v>43385</v>
       </c>
+      <c r="GW61" t="n">
+        <v>101.6</v>
+      </c>
+      <c r="GX61" t="n">
+        <v>102.45</v>
+      </c>
+      <c r="GY61" t="n">
+        <v>103.25</v>
+      </c>
+      <c r="GZ61" t="n">
+        <v>105</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -33219,6 +33819,18 @@
       <c r="GS62" t="n">
         <v>42495</v>
       </c>
+      <c r="GW62" t="n">
+        <v>101.6</v>
+      </c>
+      <c r="GX62" t="n">
+        <v>102.6</v>
+      </c>
+      <c r="GY62" t="n">
+        <v>103.25</v>
+      </c>
+      <c r="GZ62" t="n">
+        <v>105.15</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -33775,6 +34387,18 @@
       <c r="GS63" t="n">
         <v>42330</v>
       </c>
+      <c r="GW63" t="n">
+        <v>102.85</v>
+      </c>
+      <c r="GX63" t="n">
+        <v>101.8</v>
+      </c>
+      <c r="GY63" t="n">
+        <v>103.25</v>
+      </c>
+      <c r="GZ63" t="n">
+        <v>105.75</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -34289,6 +34913,18 @@
       <c r="GS64" t="n">
         <v>42470</v>
       </c>
+      <c r="GW64" t="n">
+        <v>102</v>
+      </c>
+      <c r="GX64" t="n">
+        <v>101.85</v>
+      </c>
+      <c r="GY64" t="n">
+        <v>103</v>
+      </c>
+      <c r="GZ64" t="n">
+        <v>104.15</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -34848,6 +35484,18 @@
       <c r="GS65" t="n">
         <v>42500</v>
       </c>
+      <c r="GW65" t="n">
+        <v>101.65</v>
+      </c>
+      <c r="GX65" t="n">
+        <v>102.75</v>
+      </c>
+      <c r="GY65" t="n">
+        <v>103</v>
+      </c>
+      <c r="GZ65" t="n">
+        <v>104.15</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -35401,6 +36049,18 @@
       <c r="GS66" t="n">
         <v>42850</v>
       </c>
+      <c r="GW66" t="n">
+        <v>102</v>
+      </c>
+      <c r="GX66" t="n">
+        <v>102.5</v>
+      </c>
+      <c r="GY66" t="n">
+        <v>103.5</v>
+      </c>
+      <c r="GZ66" t="n">
+        <v>104</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -35957,6 +36617,18 @@
       <c r="GS67" t="n">
         <v>42350</v>
       </c>
+      <c r="GW67" t="n">
+        <v>102</v>
+      </c>
+      <c r="GX67" t="n">
+        <v>102.25</v>
+      </c>
+      <c r="GY67" t="n">
+        <v>103.5</v>
+      </c>
+      <c r="GZ67" t="n">
+        <v>105.9</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -36495,6 +37167,18 @@
       <c r="GS68" t="n">
         <v>42560</v>
       </c>
+      <c r="GW68" t="n">
+        <v>102.3</v>
+      </c>
+      <c r="GX68" t="n">
+        <v>102.8</v>
+      </c>
+      <c r="GY68" t="n">
+        <v>103.5</v>
+      </c>
+      <c r="GZ68" t="n">
+        <v>104.35</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -37042,6 +37726,18 @@
       <c r="GU69" t="n">
         <v>732.8</v>
       </c>
+      <c r="GW69" t="n">
+        <v>101.35</v>
+      </c>
+      <c r="GX69" t="n">
+        <v>102.8</v>
+      </c>
+      <c r="GY69" t="n">
+        <v>103.5</v>
+      </c>
+      <c r="GZ69" t="n">
+        <v>104.45</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -37586,6 +38282,18 @@
       <c r="GU70" t="n">
         <v>734.5</v>
       </c>
+      <c r="GW70" t="n">
+        <v>101.2</v>
+      </c>
+      <c r="GX70" t="n">
+        <v>102.8</v>
+      </c>
+      <c r="GY70" t="n">
+        <v>103</v>
+      </c>
+      <c r="GZ70" t="n">
+        <v>104.6</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">

</xml_diff>

<commit_message>
Rellenar historia de instrumentos nuevos 2026-09-04
</commit_message>
<xml_diff>
--- a/historicos.xlsx
+++ b/historicos.xlsx
@@ -1926,6 +1926,18 @@
       <c r="GZ2" t="n">
         <v>102</v>
       </c>
+      <c r="HA2" t="n">
+        <v>100</v>
+      </c>
+      <c r="HB2" t="n">
+        <v>104.3</v>
+      </c>
+      <c r="HD2" t="n">
+        <v>102.2</v>
+      </c>
+      <c r="HE2" t="n">
+        <v>99</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -2407,6 +2419,18 @@
       <c r="GZ3" t="n">
         <v>104.75</v>
       </c>
+      <c r="HA3" t="n">
+        <v>102.2</v>
+      </c>
+      <c r="HC3" t="n">
+        <v>100.6</v>
+      </c>
+      <c r="HD3" t="n">
+        <v>104.95</v>
+      </c>
+      <c r="HE3" t="n">
+        <v>100.5</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -2891,6 +2915,18 @@
       <c r="GZ4" t="n">
         <v>103.85</v>
       </c>
+      <c r="HA4" t="n">
+        <v>102.35</v>
+      </c>
+      <c r="HC4" t="n">
+        <v>100.8</v>
+      </c>
+      <c r="HD4" t="n">
+        <v>104.9</v>
+      </c>
+      <c r="HE4" t="n">
+        <v>100.8</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -3378,6 +3414,18 @@
       <c r="GZ5" t="n">
         <v>104.1</v>
       </c>
+      <c r="HA5" t="n">
+        <v>101.65</v>
+      </c>
+      <c r="HC5" t="n">
+        <v>100.8</v>
+      </c>
+      <c r="HD5" t="n">
+        <v>104.55</v>
+      </c>
+      <c r="HE5" t="n">
+        <v>100.2</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -3874,6 +3922,18 @@
       <c r="GZ6" t="n">
         <v>104.05</v>
       </c>
+      <c r="HA6" t="n">
+        <v>102.2</v>
+      </c>
+      <c r="HC6" t="n">
+        <v>100.8</v>
+      </c>
+      <c r="HD6" t="n">
+        <v>104.8</v>
+      </c>
+      <c r="HE6" t="n">
+        <v>101.2</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -4382,6 +4442,18 @@
       <c r="GZ7" t="n">
         <v>104.15</v>
       </c>
+      <c r="HA7" t="n">
+        <v>102.55</v>
+      </c>
+      <c r="HC7" t="n">
+        <v>100.95</v>
+      </c>
+      <c r="HD7" t="n">
+        <v>105.05</v>
+      </c>
+      <c r="HE7" t="n">
+        <v>100.8</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -4884,6 +4956,18 @@
       <c r="GZ8" t="n">
         <v>104.25</v>
       </c>
+      <c r="HA8" t="n">
+        <v>101.8</v>
+      </c>
+      <c r="HC8" t="n">
+        <v>100.05</v>
+      </c>
+      <c r="HD8" t="n">
+        <v>104.05</v>
+      </c>
+      <c r="HE8" t="n">
+        <v>100.8</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -5389,6 +5473,21 @@
       <c r="GZ9" t="n">
         <v>104.45</v>
       </c>
+      <c r="HA9" t="n">
+        <v>101.8</v>
+      </c>
+      <c r="HB9" t="n">
+        <v>106.55</v>
+      </c>
+      <c r="HC9" t="n">
+        <v>100.9</v>
+      </c>
+      <c r="HD9" t="n">
+        <v>105</v>
+      </c>
+      <c r="HE9" t="n">
+        <v>100.4</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -5900,6 +5999,21 @@
       <c r="GZ10" t="n">
         <v>104.8</v>
       </c>
+      <c r="HA10" t="n">
+        <v>102.25</v>
+      </c>
+      <c r="HB10" t="n">
+        <v>107.05</v>
+      </c>
+      <c r="HC10" t="n">
+        <v>101</v>
+      </c>
+      <c r="HD10" t="n">
+        <v>105</v>
+      </c>
+      <c r="HE10" t="n">
+        <v>100.7</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -6396,6 +6510,18 @@
       <c r="GZ11" t="n">
         <v>104.25</v>
       </c>
+      <c r="HA11" t="n">
+        <v>101.95</v>
+      </c>
+      <c r="HC11" t="n">
+        <v>101</v>
+      </c>
+      <c r="HD11" t="n">
+        <v>105.15</v>
+      </c>
+      <c r="HE11" t="n">
+        <v>101.2</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -6889,6 +7015,18 @@
       <c r="GZ12" t="n">
         <v>104.2</v>
       </c>
+      <c r="HA12" t="n">
+        <v>102.3</v>
+      </c>
+      <c r="HC12" t="n">
+        <v>101</v>
+      </c>
+      <c r="HD12" t="n">
+        <v>105.15</v>
+      </c>
+      <c r="HE12" t="n">
+        <v>100.7</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -7397,6 +7535,18 @@
       <c r="GZ13" t="n">
         <v>104.35</v>
       </c>
+      <c r="HA13" t="n">
+        <v>102.9</v>
+      </c>
+      <c r="HC13" t="n">
+        <v>101.2</v>
+      </c>
+      <c r="HD13" t="n">
+        <v>105.8</v>
+      </c>
+      <c r="HE13" t="n">
+        <v>100.5</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -7905,6 +8055,18 @@
       <c r="GZ14" t="n">
         <v>104.35</v>
       </c>
+      <c r="HA14" t="n">
+        <v>102.45</v>
+      </c>
+      <c r="HC14" t="n">
+        <v>101.25</v>
+      </c>
+      <c r="HD14" t="n">
+        <v>105.1</v>
+      </c>
+      <c r="HE14" t="n">
+        <v>102.8</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -8407,6 +8569,18 @@
       <c r="GZ15" t="n">
         <v>104.5</v>
       </c>
+      <c r="HA15" t="n">
+        <v>103.4</v>
+      </c>
+      <c r="HC15" t="n">
+        <v>101.5</v>
+      </c>
+      <c r="HD15" t="n">
+        <v>105.15</v>
+      </c>
+      <c r="HE15" t="n">
+        <v>103.25</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -8927,6 +9101,18 @@
       <c r="GZ16" t="n">
         <v>104.15</v>
       </c>
+      <c r="HA16" t="n">
+        <v>103.3</v>
+      </c>
+      <c r="HC16" t="n">
+        <v>101.3</v>
+      </c>
+      <c r="HD16" t="n">
+        <v>105.2</v>
+      </c>
+      <c r="HE16" t="n">
+        <v>103.35</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -9444,6 +9630,18 @@
       <c r="GZ17" t="n">
         <v>104.35</v>
       </c>
+      <c r="HA17" t="n">
+        <v>103.5</v>
+      </c>
+      <c r="HC17" t="n">
+        <v>102</v>
+      </c>
+      <c r="HD17" t="n">
+        <v>105.7</v>
+      </c>
+      <c r="HE17" t="n">
+        <v>102.85</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -9958,6 +10156,21 @@
       <c r="GZ18" t="n">
         <v>105.35</v>
       </c>
+      <c r="HA18" t="n">
+        <v>103.4</v>
+      </c>
+      <c r="HB18" t="n">
+        <v>109.5</v>
+      </c>
+      <c r="HC18" t="n">
+        <v>101.7</v>
+      </c>
+      <c r="HD18" t="n">
+        <v>105.1</v>
+      </c>
+      <c r="HE18" t="n">
+        <v>102.75</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -10478,6 +10691,15 @@
       <c r="GZ19" t="n">
         <v>104.35</v>
       </c>
+      <c r="HA19" t="n">
+        <v>103.25</v>
+      </c>
+      <c r="HD19" t="n">
+        <v>105.4</v>
+      </c>
+      <c r="HE19" t="n">
+        <v>101.8</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -10995,6 +11217,18 @@
       <c r="GZ20" t="n">
         <v>104.45</v>
       </c>
+      <c r="HA20" t="n">
+        <v>102.3</v>
+      </c>
+      <c r="HC20" t="n">
+        <v>100.6</v>
+      </c>
+      <c r="HD20" t="n">
+        <v>105.4</v>
+      </c>
+      <c r="HE20" t="n">
+        <v>101.7</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -11515,6 +11749,18 @@
       <c r="GZ21" t="n">
         <v>104.45</v>
       </c>
+      <c r="HA21" t="n">
+        <v>102.15</v>
+      </c>
+      <c r="HC21" t="n">
+        <v>101.5</v>
+      </c>
+      <c r="HD21" t="n">
+        <v>105.7</v>
+      </c>
+      <c r="HE21" t="n">
+        <v>103.7</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -12047,6 +12293,21 @@
       <c r="GZ22" t="n">
         <v>104.3</v>
       </c>
+      <c r="HA22" t="n">
+        <v>102.65</v>
+      </c>
+      <c r="HB22" t="n">
+        <v>107.2</v>
+      </c>
+      <c r="HC22" t="n">
+        <v>101.45</v>
+      </c>
+      <c r="HD22" t="n">
+        <v>105.55</v>
+      </c>
+      <c r="HE22" t="n">
+        <v>101.9</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -12573,6 +12834,18 @@
       <c r="GZ23" t="n">
         <v>104.1</v>
       </c>
+      <c r="HA23" t="n">
+        <v>102.05</v>
+      </c>
+      <c r="HC23" t="n">
+        <v>100.55</v>
+      </c>
+      <c r="HD23" t="n">
+        <v>105.35</v>
+      </c>
+      <c r="HE23" t="n">
+        <v>103.25</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -13102,6 +13375,18 @@
       <c r="GZ24" t="n">
         <v>103.5</v>
       </c>
+      <c r="HA24" t="n">
+        <v>102.5</v>
+      </c>
+      <c r="HC24" t="n">
+        <v>101.6</v>
+      </c>
+      <c r="HD24" t="n">
+        <v>105.15</v>
+      </c>
+      <c r="HE24" t="n">
+        <v>103.2</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -13628,6 +13913,18 @@
       <c r="GZ25" t="n">
         <v>104.3</v>
       </c>
+      <c r="HA25" t="n">
+        <v>102.45</v>
+      </c>
+      <c r="HC25" t="n">
+        <v>100.65</v>
+      </c>
+      <c r="HD25" t="n">
+        <v>105.6</v>
+      </c>
+      <c r="HE25" t="n">
+        <v>102.7</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -14145,6 +14442,18 @@
       <c r="GZ26" t="n">
         <v>105.2</v>
       </c>
+      <c r="HA26" t="n">
+        <v>102.45</v>
+      </c>
+      <c r="HC26" t="n">
+        <v>100.65</v>
+      </c>
+      <c r="HD26" t="n">
+        <v>105.6</v>
+      </c>
+      <c r="HE26" t="n">
+        <v>104.2</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -14668,6 +14977,18 @@
       <c r="GZ27" t="n">
         <v>104.95</v>
       </c>
+      <c r="HA27" t="n">
+        <v>102.5</v>
+      </c>
+      <c r="HC27" t="n">
+        <v>101.75</v>
+      </c>
+      <c r="HD27" t="n">
+        <v>105.5</v>
+      </c>
+      <c r="HE27" t="n">
+        <v>103.2</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -15194,6 +15515,18 @@
       <c r="GZ28" t="n">
         <v>104.6</v>
       </c>
+      <c r="HA28" t="n">
+        <v>103</v>
+      </c>
+      <c r="HC28" t="n">
+        <v>101.65</v>
+      </c>
+      <c r="HD28" t="n">
+        <v>105</v>
+      </c>
+      <c r="HE28" t="n">
+        <v>103</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -15729,6 +16062,18 @@
       <c r="GZ29" t="n">
         <v>104.15</v>
       </c>
+      <c r="HA29" t="n">
+        <v>102.8</v>
+      </c>
+      <c r="HC29" t="n">
+        <v>101.45</v>
+      </c>
+      <c r="HD29" t="n">
+        <v>103.7</v>
+      </c>
+      <c r="HE29" t="n">
+        <v>104.1</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -16261,6 +16606,18 @@
       <c r="GZ30" t="n">
         <v>104.65</v>
       </c>
+      <c r="HA30" t="n">
+        <v>102.35</v>
+      </c>
+      <c r="HC30" t="n">
+        <v>101.8</v>
+      </c>
+      <c r="HD30" t="n">
+        <v>103.75</v>
+      </c>
+      <c r="HE30" t="n">
+        <v>102.6</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -16802,6 +17159,18 @@
       <c r="GZ31" t="n">
         <v>104.75</v>
       </c>
+      <c r="HA31" t="n">
+        <v>102.65</v>
+      </c>
+      <c r="HC31" t="n">
+        <v>101.5</v>
+      </c>
+      <c r="HD31" t="n">
+        <v>104.4</v>
+      </c>
+      <c r="HE31" t="n">
+        <v>102.8</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -17334,6 +17703,18 @@
       <c r="GZ32" t="n">
         <v>104.8</v>
       </c>
+      <c r="HA32" t="n">
+        <v>102.6</v>
+      </c>
+      <c r="HC32" t="n">
+        <v>101.2</v>
+      </c>
+      <c r="HD32" t="n">
+        <v>103</v>
+      </c>
+      <c r="HE32" t="n">
+        <v>103</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -17872,6 +18253,18 @@
       <c r="GZ33" t="n">
         <v>104.6</v>
       </c>
+      <c r="HA33" t="n">
+        <v>103.35</v>
+      </c>
+      <c r="HC33" t="n">
+        <v>100.7</v>
+      </c>
+      <c r="HD33" t="n">
+        <v>103.8</v>
+      </c>
+      <c r="HE33" t="n">
+        <v>103.25</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -18344,6 +18737,15 @@
       <c r="GZ34" t="n">
         <v>104.35</v>
       </c>
+      <c r="HC34" t="n">
+        <v>100.7</v>
+      </c>
+      <c r="HD34" t="n">
+        <v>104.5</v>
+      </c>
+      <c r="HE34" t="n">
+        <v>104</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -18885,6 +19287,18 @@
       <c r="GZ35" t="n">
         <v>104.45</v>
       </c>
+      <c r="HA35" t="n">
+        <v>102.7</v>
+      </c>
+      <c r="HC35" t="n">
+        <v>101.1</v>
+      </c>
+      <c r="HD35" t="n">
+        <v>104.05</v>
+      </c>
+      <c r="HE35" t="n">
+        <v>102.75</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -19423,6 +19837,18 @@
       <c r="GZ36" t="n">
         <v>104.75</v>
       </c>
+      <c r="HA36" t="n">
+        <v>103.3</v>
+      </c>
+      <c r="HC36" t="n">
+        <v>101.45</v>
+      </c>
+      <c r="HD36" t="n">
+        <v>104</v>
+      </c>
+      <c r="HE36" t="n">
+        <v>102.65</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -19958,6 +20384,21 @@
       <c r="GZ37" t="n">
         <v>104.6</v>
       </c>
+      <c r="HA37" t="n">
+        <v>103</v>
+      </c>
+      <c r="HB37" t="n">
+        <v>107.7</v>
+      </c>
+      <c r="HC37" t="n">
+        <v>103.9</v>
+      </c>
+      <c r="HD37" t="n">
+        <v>103.8</v>
+      </c>
+      <c r="HE37" t="n">
+        <v>102.9</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -20496,6 +20937,21 @@
       <c r="GZ38" t="n">
         <v>104.8</v>
       </c>
+      <c r="HA38" t="n">
+        <v>103.3</v>
+      </c>
+      <c r="HB38" t="n">
+        <v>107.9</v>
+      </c>
+      <c r="HC38" t="n">
+        <v>102.45</v>
+      </c>
+      <c r="HD38" t="n">
+        <v>103.7</v>
+      </c>
+      <c r="HE38" t="n">
+        <v>102.5</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -21049,6 +21505,18 @@
       <c r="GZ39" t="n">
         <v>105.4</v>
       </c>
+      <c r="HA39" t="n">
+        <v>103.75</v>
+      </c>
+      <c r="HC39" t="n">
+        <v>102.5</v>
+      </c>
+      <c r="HD39" t="n">
+        <v>103.85</v>
+      </c>
+      <c r="HE39" t="n">
+        <v>102.85</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -21593,6 +22061,18 @@
       <c r="GZ40" t="n">
         <v>105</v>
       </c>
+      <c r="HA40" t="n">
+        <v>103.8</v>
+      </c>
+      <c r="HC40" t="n">
+        <v>102.5</v>
+      </c>
+      <c r="HD40" t="n">
+        <v>103.85</v>
+      </c>
+      <c r="HE40" t="n">
+        <v>102.8</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -22137,6 +22617,18 @@
       <c r="GZ41" t="n">
         <v>104.85</v>
       </c>
+      <c r="HA41" t="n">
+        <v>103.75</v>
+      </c>
+      <c r="HC41" t="n">
+        <v>102.8</v>
+      </c>
+      <c r="HD41" t="n">
+        <v>103.85</v>
+      </c>
+      <c r="HE41" t="n">
+        <v>103.3</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -22681,6 +23173,21 @@
       <c r="GZ42" t="n">
         <v>104.95</v>
       </c>
+      <c r="HA42" t="n">
+        <v>103.5</v>
+      </c>
+      <c r="HB42" t="n">
+        <v>104</v>
+      </c>
+      <c r="HC42" t="n">
+        <v>103.5</v>
+      </c>
+      <c r="HD42" t="n">
+        <v>103.9</v>
+      </c>
+      <c r="HE42" t="n">
+        <v>102.25</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -23222,6 +23729,18 @@
       <c r="GZ43" t="n">
         <v>104.9</v>
       </c>
+      <c r="HA43" t="n">
+        <v>103.5</v>
+      </c>
+      <c r="HC43" t="n">
+        <v>103.5</v>
+      </c>
+      <c r="HD43" t="n">
+        <v>104.1</v>
+      </c>
+      <c r="HE43" t="n">
+        <v>102.7</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -23775,6 +24294,21 @@
       <c r="GZ44" t="n">
         <v>105.4</v>
       </c>
+      <c r="HA44" t="n">
+        <v>103.7</v>
+      </c>
+      <c r="HB44" t="n">
+        <v>104</v>
+      </c>
+      <c r="HC44" t="n">
+        <v>103.3</v>
+      </c>
+      <c r="HD44" t="n">
+        <v>104.7</v>
+      </c>
+      <c r="HE44" t="n">
+        <v>103.4</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -24328,6 +24862,21 @@
       <c r="GZ45" t="n">
         <v>104.9</v>
       </c>
+      <c r="HA45" t="n">
+        <v>103.05</v>
+      </c>
+      <c r="HB45" t="n">
+        <v>104.1</v>
+      </c>
+      <c r="HC45" t="n">
+        <v>103.1</v>
+      </c>
+      <c r="HD45" t="n">
+        <v>104.6</v>
+      </c>
+      <c r="HE45" t="n">
+        <v>103.5</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -24878,6 +25427,21 @@
       <c r="GZ46" t="n">
         <v>104.95</v>
       </c>
+      <c r="HA46" t="n">
+        <v>103.05</v>
+      </c>
+      <c r="HB46" t="n">
+        <v>103.5</v>
+      </c>
+      <c r="HC46" t="n">
+        <v>103.3</v>
+      </c>
+      <c r="HD46" t="n">
+        <v>104.65</v>
+      </c>
+      <c r="HE46" t="n">
+        <v>104</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -25428,6 +25992,21 @@
       <c r="GZ47" t="n">
         <v>104.95</v>
       </c>
+      <c r="HA47" t="n">
+        <v>103.35</v>
+      </c>
+      <c r="HB47" t="n">
+        <v>103.9</v>
+      </c>
+      <c r="HC47" t="n">
+        <v>105</v>
+      </c>
+      <c r="HD47" t="n">
+        <v>104.65</v>
+      </c>
+      <c r="HE47" t="n">
+        <v>103.5</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="3" t="n">
@@ -25967,6 +26546,21 @@
       <c r="GZ48" t="n">
         <v>104.6</v>
       </c>
+      <c r="HA48" t="n">
+        <v>103.4</v>
+      </c>
+      <c r="HB48" t="n">
+        <v>104.1</v>
+      </c>
+      <c r="HC48" t="n">
+        <v>102.5</v>
+      </c>
+      <c r="HD48" t="n">
+        <v>104.5</v>
+      </c>
+      <c r="HE48" t="n">
+        <v>104.35</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="3" t="n">
@@ -26517,6 +27111,18 @@
       </c>
       <c r="GZ49" t="n">
         <v>104.95</v>
+      </c>
+      <c r="HA49" t="n">
+        <v>102.85</v>
+      </c>
+      <c r="HB49" t="n">
+        <v>104.5</v>
+      </c>
+      <c r="HD49" t="n">
+        <v>104.2</v>
+      </c>
+      <c r="HE49" t="n">
+        <v>103.45</v>
       </c>
     </row>
     <row r="50">
@@ -27086,6 +27692,18 @@
       <c r="GZ50" t="n">
         <v>104.95</v>
       </c>
+      <c r="HA50" t="n">
+        <v>103.45</v>
+      </c>
+      <c r="HC50" t="n">
+        <v>103.05</v>
+      </c>
+      <c r="HD50" t="n">
+        <v>104.25</v>
+      </c>
+      <c r="HE50" t="n">
+        <v>104.15</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -27645,6 +28263,21 @@
       <c r="GZ51" t="n">
         <v>105</v>
       </c>
+      <c r="HA51" t="n">
+        <v>103.8</v>
+      </c>
+      <c r="HB51" t="n">
+        <v>105</v>
+      </c>
+      <c r="HC51" t="n">
+        <v>104</v>
+      </c>
+      <c r="HD51" t="n">
+        <v>105</v>
+      </c>
+      <c r="HE51" t="n">
+        <v>102.9</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -28204,6 +28837,18 @@
       <c r="GZ52" t="n">
         <v>104.85</v>
       </c>
+      <c r="HA52" t="n">
+        <v>103.85</v>
+      </c>
+      <c r="HC52" t="n">
+        <v>102.55</v>
+      </c>
+      <c r="HD52" t="n">
+        <v>104.75</v>
+      </c>
+      <c r="HE52" t="n">
+        <v>102.5</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="4" t="n">
@@ -28770,6 +29415,18 @@
       <c r="GZ53" t="n">
         <v>105</v>
       </c>
+      <c r="HA53" t="n">
+        <v>103.85</v>
+      </c>
+      <c r="HC53" t="n">
+        <v>103.45</v>
+      </c>
+      <c r="HD53" t="n">
+        <v>104.95</v>
+      </c>
+      <c r="HE53" t="n">
+        <v>102.6</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="3" t="n">
@@ -29332,6 +29989,18 @@
       </c>
       <c r="GZ54" t="n">
         <v>105</v>
+      </c>
+      <c r="HA54" t="n">
+        <v>103.15</v>
+      </c>
+      <c r="HC54" t="n">
+        <v>103.4</v>
+      </c>
+      <c r="HD54" t="n">
+        <v>104.35</v>
+      </c>
+      <c r="HE54" t="n">
+        <v>102.35</v>
       </c>
     </row>
     <row r="55">
@@ -29898,6 +30567,18 @@
       <c r="GZ55" t="n">
         <v>105.45</v>
       </c>
+      <c r="HA55" t="n">
+        <v>103.2</v>
+      </c>
+      <c r="HC55" t="n">
+        <v>104.9</v>
+      </c>
+      <c r="HD55" t="n">
+        <v>104.6</v>
+      </c>
+      <c r="HE55" t="n">
+        <v>102.8</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -30466,6 +31147,18 @@
       <c r="GZ56" t="n">
         <v>105</v>
       </c>
+      <c r="HA56" t="n">
+        <v>103.8</v>
+      </c>
+      <c r="HC56" t="n">
+        <v>104.65</v>
+      </c>
+      <c r="HD56" t="n">
+        <v>104.3</v>
+      </c>
+      <c r="HE56" t="n">
+        <v>104.45</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -31028,6 +31721,18 @@
       <c r="GZ57" t="n">
         <v>105.1</v>
       </c>
+      <c r="HA57" t="n">
+        <v>103</v>
+      </c>
+      <c r="HC57" t="n">
+        <v>104.75</v>
+      </c>
+      <c r="HD57" t="n">
+        <v>104.05</v>
+      </c>
+      <c r="HE57" t="n">
+        <v>104.45</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -31587,6 +32292,21 @@
       <c r="GZ58" t="n">
         <v>105</v>
       </c>
+      <c r="HA58" t="n">
+        <v>103.7</v>
+      </c>
+      <c r="HB58" t="n">
+        <v>105</v>
+      </c>
+      <c r="HC58" t="n">
+        <v>102.5</v>
+      </c>
+      <c r="HD58" t="n">
+        <v>104.2</v>
+      </c>
+      <c r="HE58" t="n">
+        <v>103.15</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -32152,6 +32872,18 @@
       <c r="GZ59" t="n">
         <v>105.2</v>
       </c>
+      <c r="HA59" t="n">
+        <v>103.7</v>
+      </c>
+      <c r="HC59" t="n">
+        <v>102.5</v>
+      </c>
+      <c r="HD59" t="n">
+        <v>104.35</v>
+      </c>
+      <c r="HE59" t="n">
+        <v>103.15</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -32723,6 +33455,18 @@
       <c r="GZ60" t="n">
         <v>105.5</v>
       </c>
+      <c r="HA60" t="n">
+        <v>103.2</v>
+      </c>
+      <c r="HC60" t="n">
+        <v>102.9</v>
+      </c>
+      <c r="HD60" t="n">
+        <v>104.15</v>
+      </c>
+      <c r="HE60" t="n">
+        <v>103.2</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -33291,6 +34035,21 @@
       <c r="GZ61" t="n">
         <v>105</v>
       </c>
+      <c r="HA61" t="n">
+        <v>103.2</v>
+      </c>
+      <c r="HB61" t="n">
+        <v>104.85</v>
+      </c>
+      <c r="HC61" t="n">
+        <v>103</v>
+      </c>
+      <c r="HD61" t="n">
+        <v>104.1</v>
+      </c>
+      <c r="HE61" t="n">
+        <v>102.6</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -33856,6 +34615,21 @@
       <c r="GZ62" t="n">
         <v>105.15</v>
       </c>
+      <c r="HA62" t="n">
+        <v>103.2</v>
+      </c>
+      <c r="HB62" t="n">
+        <v>105.2</v>
+      </c>
+      <c r="HC62" t="n">
+        <v>102.4</v>
+      </c>
+      <c r="HD62" t="n">
+        <v>103.7</v>
+      </c>
+      <c r="HE62" t="n">
+        <v>102.35</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -34424,6 +35198,18 @@
       <c r="GZ63" t="n">
         <v>105.75</v>
       </c>
+      <c r="HA63" t="n">
+        <v>103.1</v>
+      </c>
+      <c r="HC63" t="n">
+        <v>102.5</v>
+      </c>
+      <c r="HD63" t="n">
+        <v>104.4</v>
+      </c>
+      <c r="HE63" t="n">
+        <v>103</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -34950,6 +35736,18 @@
       <c r="GZ64" t="n">
         <v>104.15</v>
       </c>
+      <c r="HA64" t="n">
+        <v>103</v>
+      </c>
+      <c r="HC64" t="n">
+        <v>103</v>
+      </c>
+      <c r="HD64" t="n">
+        <v>103.8</v>
+      </c>
+      <c r="HE64" t="n">
+        <v>102.95</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -35521,6 +36319,18 @@
       <c r="GZ65" t="n">
         <v>104.15</v>
       </c>
+      <c r="HA65" t="n">
+        <v>103</v>
+      </c>
+      <c r="HC65" t="n">
+        <v>102.45</v>
+      </c>
+      <c r="HD65" t="n">
+        <v>104.3</v>
+      </c>
+      <c r="HE65" t="n">
+        <v>102.95</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -36086,6 +36896,21 @@
       <c r="GZ66" t="n">
         <v>104</v>
       </c>
+      <c r="HA66" t="n">
+        <v>103.1</v>
+      </c>
+      <c r="HB66" t="n">
+        <v>104.3</v>
+      </c>
+      <c r="HC66" t="n">
+        <v>102.7</v>
+      </c>
+      <c r="HD66" t="n">
+        <v>104</v>
+      </c>
+      <c r="HE66" t="n">
+        <v>103</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -36654,6 +37479,21 @@
       <c r="GZ67" t="n">
         <v>105.9</v>
       </c>
+      <c r="HA67" t="n">
+        <v>102.85</v>
+      </c>
+      <c r="HB67" t="n">
+        <v>105.05</v>
+      </c>
+      <c r="HC67" t="n">
+        <v>103.05</v>
+      </c>
+      <c r="HD67" t="n">
+        <v>104.85</v>
+      </c>
+      <c r="HE67" t="n">
+        <v>102.65</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -37204,6 +38044,21 @@
       <c r="GZ68" t="n">
         <v>104.35</v>
       </c>
+      <c r="HA68" t="n">
+        <v>103.25</v>
+      </c>
+      <c r="HB68" t="n">
+        <v>104.6</v>
+      </c>
+      <c r="HC68" t="n">
+        <v>102.95</v>
+      </c>
+      <c r="HD68" t="n">
+        <v>105.05</v>
+      </c>
+      <c r="HE68" t="n">
+        <v>102.85</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -37763,6 +38618,18 @@
       <c r="GZ69" t="n">
         <v>104.45</v>
       </c>
+      <c r="HA69" t="n">
+        <v>103.2</v>
+      </c>
+      <c r="HC69" t="n">
+        <v>103.1</v>
+      </c>
+      <c r="HD69" t="n">
+        <v>104.2</v>
+      </c>
+      <c r="HE69" t="n">
+        <v>103.05</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -38319,6 +39186,18 @@
       <c r="GZ70" t="n">
         <v>104.6</v>
       </c>
+      <c r="HA70" t="n">
+        <v>102.85</v>
+      </c>
+      <c r="HC70" t="n">
+        <v>103</v>
+      </c>
+      <c r="HD70" t="n">
+        <v>103.8</v>
+      </c>
+      <c r="HE70" t="n">
+        <v>103</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -38881,6 +39760,18 @@
       <c r="GZ71" t="n">
         <v>104.3</v>
       </c>
+      <c r="HA71" t="n">
+        <v>102.9</v>
+      </c>
+      <c r="HC71" t="n">
+        <v>102.4</v>
+      </c>
+      <c r="HD71" t="n">
+        <v>104</v>
+      </c>
+      <c r="HE71" t="n">
+        <v>102.95</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -39443,6 +40334,18 @@
       <c r="GZ72" t="n">
         <v>104</v>
       </c>
+      <c r="HA72" t="n">
+        <v>103.25</v>
+      </c>
+      <c r="HC72" t="n">
+        <v>102.85</v>
+      </c>
+      <c r="HD72" t="n">
+        <v>104.9</v>
+      </c>
+      <c r="HE72" t="n">
+        <v>104</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">

</xml_diff>

<commit_message>
Rellenar historia de instrumentos nuevos 2026-09-08
</commit_message>
<xml_diff>
--- a/historicos.xlsx
+++ b/historicos.xlsx
@@ -1963,6 +1963,12 @@
       <c r="HE2" t="n">
         <v>99</v>
       </c>
+      <c r="HI2" t="n">
+        <v>94.5</v>
+      </c>
+      <c r="HJ2" t="n">
+        <v>105.35</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -2456,6 +2462,12 @@
       <c r="HE3" t="n">
         <v>100.5</v>
       </c>
+      <c r="HI3" t="n">
+        <v>103</v>
+      </c>
+      <c r="HJ3" t="n">
+        <v>106.75</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -2952,6 +2964,12 @@
       <c r="HE4" t="n">
         <v>100.8</v>
       </c>
+      <c r="HI4" t="n">
+        <v>101.75</v>
+      </c>
+      <c r="HJ4" t="n">
+        <v>106.15</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -3451,6 +3469,12 @@
       <c r="HE5" t="n">
         <v>100.2</v>
       </c>
+      <c r="HI5" t="n">
+        <v>102</v>
+      </c>
+      <c r="HJ5" t="n">
+        <v>106.4</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -3959,6 +3983,12 @@
       <c r="HE6" t="n">
         <v>101.2</v>
       </c>
+      <c r="HI6" t="n">
+        <v>102.6</v>
+      </c>
+      <c r="HJ6" t="n">
+        <v>107</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -4479,6 +4509,12 @@
       <c r="HE7" t="n">
         <v>100.8</v>
       </c>
+      <c r="HI7" t="n">
+        <v>103.2</v>
+      </c>
+      <c r="HJ7" t="n">
+        <v>106.2</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -4993,6 +5029,12 @@
       <c r="HE8" t="n">
         <v>100.8</v>
       </c>
+      <c r="HI8" t="n">
+        <v>103</v>
+      </c>
+      <c r="HJ8" t="n">
+        <v>105.8</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -5513,6 +5555,12 @@
       <c r="HE9" t="n">
         <v>100.4</v>
       </c>
+      <c r="HI9" t="n">
+        <v>102.85</v>
+      </c>
+      <c r="HJ9" t="n">
+        <v>106.2</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -6039,6 +6087,12 @@
       <c r="HE10" t="n">
         <v>100.7</v>
       </c>
+      <c r="HI10" t="n">
+        <v>103.55</v>
+      </c>
+      <c r="HJ10" t="n">
+        <v>106.9</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -6547,6 +6601,12 @@
       <c r="HE11" t="n">
         <v>101.2</v>
       </c>
+      <c r="HI11" t="n">
+        <v>101.65</v>
+      </c>
+      <c r="HJ11" t="n">
+        <v>106.85</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -7052,6 +7112,12 @@
       <c r="HE12" t="n">
         <v>100.7</v>
       </c>
+      <c r="HI12" t="n">
+        <v>103</v>
+      </c>
+      <c r="HJ12" t="n">
+        <v>106.3</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -7572,6 +7638,12 @@
       <c r="HE13" t="n">
         <v>100.5</v>
       </c>
+      <c r="HI13" t="n">
+        <v>103</v>
+      </c>
+      <c r="HJ13" t="n">
+        <v>107.7</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -8092,6 +8164,12 @@
       <c r="HE14" t="n">
         <v>102.8</v>
       </c>
+      <c r="HI14" t="n">
+        <v>103.7</v>
+      </c>
+      <c r="HJ14" t="n">
+        <v>107.2</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -8606,6 +8684,12 @@
       <c r="HE15" t="n">
         <v>103.25</v>
       </c>
+      <c r="HI15" t="n">
+        <v>103.2</v>
+      </c>
+      <c r="HJ15" t="n">
+        <v>108.5</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -9138,6 +9222,12 @@
       <c r="HE16" t="n">
         <v>103.35</v>
       </c>
+      <c r="HI16" t="n">
+        <v>103.8</v>
+      </c>
+      <c r="HJ16" t="n">
+        <v>108.45</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -9667,6 +9757,12 @@
       <c r="HE17" t="n">
         <v>102.85</v>
       </c>
+      <c r="HI17" t="n">
+        <v>103.2</v>
+      </c>
+      <c r="HJ17" t="n">
+        <v>107.5</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -10196,6 +10292,12 @@
       <c r="HE18" t="n">
         <v>102.75</v>
       </c>
+      <c r="HI18" t="n">
+        <v>103.95</v>
+      </c>
+      <c r="HJ18" t="n">
+        <v>107.15</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -10725,6 +10827,12 @@
       <c r="HE19" t="n">
         <v>101.8</v>
       </c>
+      <c r="HI19" t="n">
+        <v>102.5</v>
+      </c>
+      <c r="HJ19" t="n">
+        <v>106.9</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -11254,6 +11362,12 @@
       <c r="HE20" t="n">
         <v>101.7</v>
       </c>
+      <c r="HI20" t="n">
+        <v>102.95</v>
+      </c>
+      <c r="HJ20" t="n">
+        <v>107.2</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -11786,6 +11900,12 @@
       <c r="HE21" t="n">
         <v>103.7</v>
       </c>
+      <c r="HI21" t="n">
+        <v>103.4</v>
+      </c>
+      <c r="HJ21" t="n">
+        <v>106.9</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -12333,6 +12453,12 @@
       <c r="HE22" t="n">
         <v>101.9</v>
       </c>
+      <c r="HI22" t="n">
+        <v>101.1</v>
+      </c>
+      <c r="HJ22" t="n">
+        <v>107.7</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -12871,6 +12997,12 @@
       <c r="HE23" t="n">
         <v>103.25</v>
       </c>
+      <c r="HI23" t="n">
+        <v>102.7</v>
+      </c>
+      <c r="HJ23" t="n">
+        <v>107.75</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -13412,6 +13544,12 @@
       <c r="HE24" t="n">
         <v>103.2</v>
       </c>
+      <c r="HI24" t="n">
+        <v>103</v>
+      </c>
+      <c r="HJ24" t="n">
+        <v>107.8</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -13950,6 +14088,12 @@
       <c r="HE25" t="n">
         <v>102.7</v>
       </c>
+      <c r="HI25" t="n">
+        <v>103.05</v>
+      </c>
+      <c r="HJ25" t="n">
+        <v>108.85</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -14479,6 +14623,12 @@
       <c r="HE26" t="n">
         <v>104.2</v>
       </c>
+      <c r="HI26" t="n">
+        <v>103</v>
+      </c>
+      <c r="HJ26" t="n">
+        <v>107.75</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -15014,6 +15164,12 @@
       <c r="HE27" t="n">
         <v>103.2</v>
       </c>
+      <c r="HI27" t="n">
+        <v>103</v>
+      </c>
+      <c r="HJ27" t="n">
+        <v>108.35</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -15552,6 +15708,12 @@
       <c r="HE28" t="n">
         <v>103</v>
       </c>
+      <c r="HI28" t="n">
+        <v>103</v>
+      </c>
+      <c r="HJ28" t="n">
+        <v>107.9</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -16099,6 +16261,12 @@
       <c r="HE29" t="n">
         <v>104.1</v>
       </c>
+      <c r="HI29" t="n">
+        <v>103</v>
+      </c>
+      <c r="HJ29" t="n">
+        <v>108.6</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -16643,6 +16811,12 @@
       <c r="HE30" t="n">
         <v>102.6</v>
       </c>
+      <c r="HI30" t="n">
+        <v>103.85</v>
+      </c>
+      <c r="HJ30" t="n">
+        <v>107.5</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -17196,6 +17370,12 @@
       <c r="HE31" t="n">
         <v>102.8</v>
       </c>
+      <c r="HI31" t="n">
+        <v>103.85</v>
+      </c>
+      <c r="HJ31" t="n">
+        <v>107.2</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -17740,6 +17920,12 @@
       <c r="HE32" t="n">
         <v>103</v>
       </c>
+      <c r="HI32" t="n">
+        <v>103.9</v>
+      </c>
+      <c r="HJ32" t="n">
+        <v>107.4</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -18290,6 +18476,12 @@
       <c r="HE33" t="n">
         <v>103.25</v>
       </c>
+      <c r="HI33" t="n">
+        <v>103.8</v>
+      </c>
+      <c r="HJ33" t="n">
+        <v>107.25</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -18771,6 +18963,12 @@
       <c r="HE34" t="n">
         <v>104</v>
       </c>
+      <c r="HI34" t="n">
+        <v>103.9</v>
+      </c>
+      <c r="HJ34" t="n">
+        <v>107.5</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -19324,6 +19522,15 @@
       <c r="HE35" t="n">
         <v>102.75</v>
       </c>
+      <c r="HF35" t="n">
+        <v>106.25</v>
+      </c>
+      <c r="HI35" t="n">
+        <v>103.8</v>
+      </c>
+      <c r="HJ35" t="n">
+        <v>107.45</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -19874,6 +20081,15 @@
       <c r="HE36" t="n">
         <v>102.65</v>
       </c>
+      <c r="HF36" t="n">
+        <v>106.3</v>
+      </c>
+      <c r="HI36" t="n">
+        <v>103.9</v>
+      </c>
+      <c r="HJ36" t="n">
+        <v>107.7</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -20424,6 +20640,15 @@
       <c r="HE37" t="n">
         <v>102.9</v>
       </c>
+      <c r="HF37" t="n">
+        <v>106.35</v>
+      </c>
+      <c r="HI37" t="n">
+        <v>103.8</v>
+      </c>
+      <c r="HJ37" t="n">
+        <v>108</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -20977,6 +21202,15 @@
       <c r="HE38" t="n">
         <v>102.5</v>
       </c>
+      <c r="HH38" t="n">
+        <v>100</v>
+      </c>
+      <c r="HI38" t="n">
+        <v>103.8</v>
+      </c>
+      <c r="HJ38" t="n">
+        <v>108.1</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -21542,6 +21776,18 @@
       <c r="HE39" t="n">
         <v>102.85</v>
       </c>
+      <c r="HF39" t="n">
+        <v>106.45</v>
+      </c>
+      <c r="HH39" t="n">
+        <v>100</v>
+      </c>
+      <c r="HI39" t="n">
+        <v>104</v>
+      </c>
+      <c r="HJ39" t="n">
+        <v>108.4</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -22098,6 +22344,12 @@
       <c r="HE40" t="n">
         <v>102.8</v>
       </c>
+      <c r="HI40" t="n">
+        <v>104.1</v>
+      </c>
+      <c r="HJ40" t="n">
+        <v>108.1</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -22654,6 +22906,12 @@
       <c r="HE41" t="n">
         <v>103.3</v>
       </c>
+      <c r="HI41" t="n">
+        <v>104.05</v>
+      </c>
+      <c r="HJ41" t="n">
+        <v>108.35</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -23213,6 +23471,12 @@
       <c r="HE42" t="n">
         <v>102.25</v>
       </c>
+      <c r="HI42" t="n">
+        <v>101.5</v>
+      </c>
+      <c r="HJ42" t="n">
+        <v>106.5</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -23766,6 +24030,15 @@
       <c r="HE43" t="n">
         <v>102.7</v>
       </c>
+      <c r="HH43" t="n">
+        <v>96.99999999999999</v>
+      </c>
+      <c r="HI43" t="n">
+        <v>100.6</v>
+      </c>
+      <c r="HJ43" t="n">
+        <v>107.4</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -24334,6 +24607,18 @@
       <c r="HE44" t="n">
         <v>103.4</v>
       </c>
+      <c r="HF44" t="n">
+        <v>106.7</v>
+      </c>
+      <c r="HH44" t="n">
+        <v>98.5</v>
+      </c>
+      <c r="HI44" t="n">
+        <v>100.95</v>
+      </c>
+      <c r="HJ44" t="n">
+        <v>106.3</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -24902,6 +25187,15 @@
       <c r="HE45" t="n">
         <v>103.5</v>
       </c>
+      <c r="HH45" t="n">
+        <v>98.00000000000001</v>
+      </c>
+      <c r="HI45" t="n">
+        <v>101.2</v>
+      </c>
+      <c r="HJ45" t="n">
+        <v>105.2</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -25467,6 +25761,18 @@
       <c r="HE46" t="n">
         <v>104</v>
       </c>
+      <c r="HF46" t="n">
+        <v>105.6</v>
+      </c>
+      <c r="HH46" t="n">
+        <v>98.51000000000001</v>
+      </c>
+      <c r="HI46" t="n">
+        <v>100.25</v>
+      </c>
+      <c r="HJ46" t="n">
+        <v>106.3</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -26032,6 +26338,15 @@
       <c r="HE47" t="n">
         <v>103.5</v>
       </c>
+      <c r="HH47" t="n">
+        <v>100</v>
+      </c>
+      <c r="HI47" t="n">
+        <v>100</v>
+      </c>
+      <c r="HJ47" t="n">
+        <v>105.4</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="3" t="n">
@@ -26586,6 +26901,12 @@
       <c r="HE48" t="n">
         <v>104.35</v>
       </c>
+      <c r="HI48" t="n">
+        <v>101</v>
+      </c>
+      <c r="HJ48" t="n">
+        <v>104.9</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="3" t="n">
@@ -27148,6 +27469,12 @@
       </c>
       <c r="HE49" t="n">
         <v>103.45</v>
+      </c>
+      <c r="HI49" t="n">
+        <v>101.95</v>
+      </c>
+      <c r="HJ49" t="n">
+        <v>105.05</v>
       </c>
     </row>
     <row r="50">
@@ -27729,6 +28056,15 @@
       <c r="HE50" t="n">
         <v>104.15</v>
       </c>
+      <c r="HF50" t="n">
+        <v>106.45</v>
+      </c>
+      <c r="HI50" t="n">
+        <v>101.95</v>
+      </c>
+      <c r="HJ50" t="n">
+        <v>105.9</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -28303,6 +28639,12 @@
       <c r="HE51" t="n">
         <v>102.9</v>
       </c>
+      <c r="HI51" t="n">
+        <v>101.85</v>
+      </c>
+      <c r="HJ51" t="n">
+        <v>105.9</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -28874,6 +29216,15 @@
       <c r="HE52" t="n">
         <v>102.5</v>
       </c>
+      <c r="HF52" t="n">
+        <v>106.8</v>
+      </c>
+      <c r="HI52" t="n">
+        <v>101.85</v>
+      </c>
+      <c r="HJ52" t="n">
+        <v>105.75</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="4" t="n">
@@ -29452,6 +29803,12 @@
       <c r="HE53" t="n">
         <v>102.6</v>
       </c>
+      <c r="HI53" t="n">
+        <v>101.85</v>
+      </c>
+      <c r="HJ53" t="n">
+        <v>105.4</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="3" t="n">
@@ -30026,6 +30383,15 @@
       </c>
       <c r="HE54" t="n">
         <v>102.35</v>
+      </c>
+      <c r="HF54" t="n">
+        <v>106.35</v>
+      </c>
+      <c r="HI54" t="n">
+        <v>102.3</v>
+      </c>
+      <c r="HJ54" t="n">
+        <v>106.65</v>
       </c>
     </row>
     <row r="55">
@@ -30604,6 +30970,12 @@
       <c r="HE55" t="n">
         <v>102.8</v>
       </c>
+      <c r="HI55" t="n">
+        <v>102.1</v>
+      </c>
+      <c r="HJ55" t="n">
+        <v>105.8</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -31184,6 +31556,15 @@
       <c r="HE56" t="n">
         <v>104.45</v>
       </c>
+      <c r="HF56" t="n">
+        <v>106.3</v>
+      </c>
+      <c r="HI56" t="n">
+        <v>102.25</v>
+      </c>
+      <c r="HJ56" t="n">
+        <v>105.45</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -31758,6 +32139,12 @@
       <c r="HE57" t="n">
         <v>104.45</v>
       </c>
+      <c r="HI57" t="n">
+        <v>102</v>
+      </c>
+      <c r="HJ57" t="n">
+        <v>104.8</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -32332,6 +32719,12 @@
       <c r="HE58" t="n">
         <v>103.15</v>
       </c>
+      <c r="HI58" t="n">
+        <v>101.5</v>
+      </c>
+      <c r="HJ58" t="n">
+        <v>105.7</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -32909,6 +33302,18 @@
       <c r="HE59" t="n">
         <v>103.15</v>
       </c>
+      <c r="HF59" t="n">
+        <v>106.3</v>
+      </c>
+      <c r="HH59" t="n">
+        <v>100.5</v>
+      </c>
+      <c r="HI59" t="n">
+        <v>101.5</v>
+      </c>
+      <c r="HJ59" t="n">
+        <v>105.4</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -33492,6 +33897,12 @@
       <c r="HE60" t="n">
         <v>103.2</v>
       </c>
+      <c r="HI60" t="n">
+        <v>101.85</v>
+      </c>
+      <c r="HJ60" t="n">
+        <v>105.7</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -34075,6 +34486,15 @@
       <c r="HE61" t="n">
         <v>102.6</v>
       </c>
+      <c r="HF61" t="n">
+        <v>106.2</v>
+      </c>
+      <c r="HI61" t="n">
+        <v>101.7</v>
+      </c>
+      <c r="HJ61" t="n">
+        <v>105</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -34655,6 +35075,18 @@
       <c r="HE62" t="n">
         <v>102.35</v>
       </c>
+      <c r="HF62" t="n">
+        <v>106.2</v>
+      </c>
+      <c r="HH62" t="n">
+        <v>100.6</v>
+      </c>
+      <c r="HI62" t="n">
+        <v>101.9</v>
+      </c>
+      <c r="HJ62" t="n">
+        <v>104.7</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -35235,6 +35667,18 @@
       <c r="HE63" t="n">
         <v>103</v>
       </c>
+      <c r="HF63" t="n">
+        <v>106.25</v>
+      </c>
+      <c r="HG63" t="n">
+        <v>99.95000000000002</v>
+      </c>
+      <c r="HI63" t="n">
+        <v>101.9</v>
+      </c>
+      <c r="HJ63" t="n">
+        <v>104.7</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -35773,6 +36217,15 @@
       <c r="HE64" t="n">
         <v>102.95</v>
       </c>
+      <c r="HG64" t="n">
+        <v>99.5</v>
+      </c>
+      <c r="HI64" t="n">
+        <v>102</v>
+      </c>
+      <c r="HJ64" t="n">
+        <v>104.5</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -36356,6 +36809,21 @@
       <c r="HE65" t="n">
         <v>102.95</v>
       </c>
+      <c r="HF65" t="n">
+        <v>105.95</v>
+      </c>
+      <c r="HG65" t="n">
+        <v>99.59999999999998</v>
+      </c>
+      <c r="HH65" t="n">
+        <v>99.20000000000002</v>
+      </c>
+      <c r="HI65" t="n">
+        <v>101.9</v>
+      </c>
+      <c r="HJ65" t="n">
+        <v>104.1</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -36936,6 +37404,15 @@
       <c r="HE66" t="n">
         <v>103</v>
       </c>
+      <c r="HG66" t="n">
+        <v>99.59999999999998</v>
+      </c>
+      <c r="HI66" t="n">
+        <v>101.9</v>
+      </c>
+      <c r="HJ66" t="n">
+        <v>104.35</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -37519,6 +37996,18 @@
       <c r="HE67" t="n">
         <v>102.65</v>
       </c>
+      <c r="HG67" t="n">
+        <v>100</v>
+      </c>
+      <c r="HH67" t="n">
+        <v>100.5</v>
+      </c>
+      <c r="HI67" t="n">
+        <v>101.75</v>
+      </c>
+      <c r="HJ67" t="n">
+        <v>104</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -38084,6 +38573,18 @@
       <c r="HE68" t="n">
         <v>102.85</v>
       </c>
+      <c r="HF68" t="n">
+        <v>105.9</v>
+      </c>
+      <c r="HG68" t="n">
+        <v>100</v>
+      </c>
+      <c r="HI68" t="n">
+        <v>101.8</v>
+      </c>
+      <c r="HJ68" t="n">
+        <v>104.9</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -38655,6 +39156,18 @@
       <c r="HE69" t="n">
         <v>103.05</v>
       </c>
+      <c r="HF69" t="n">
+        <v>105.8</v>
+      </c>
+      <c r="HG69" t="n">
+        <v>99.75000000000001</v>
+      </c>
+      <c r="HI69" t="n">
+        <v>101.2</v>
+      </c>
+      <c r="HJ69" t="n">
+        <v>104.95</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -39223,6 +39736,21 @@
       <c r="HE70" t="n">
         <v>103</v>
       </c>
+      <c r="HF70" t="n">
+        <v>104.5</v>
+      </c>
+      <c r="HG70" t="n">
+        <v>100.25</v>
+      </c>
+      <c r="HH70" t="n">
+        <v>100.6</v>
+      </c>
+      <c r="HI70" t="n">
+        <v>101.8</v>
+      </c>
+      <c r="HJ70" t="n">
+        <v>104.9</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -39797,6 +40325,18 @@
       <c r="HE71" t="n">
         <v>102.95</v>
       </c>
+      <c r="HG71" t="n">
+        <v>100</v>
+      </c>
+      <c r="HH71" t="n">
+        <v>100.6</v>
+      </c>
+      <c r="HI71" t="n">
+        <v>101.6</v>
+      </c>
+      <c r="HJ71" t="n">
+        <v>105</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -40371,6 +40911,18 @@
       <c r="HE72" t="n">
         <v>104</v>
       </c>
+      <c r="HF72" t="n">
+        <v>104.25</v>
+      </c>
+      <c r="HG72" t="n">
+        <v>100</v>
+      </c>
+      <c r="HI72" t="n">
+        <v>101</v>
+      </c>
+      <c r="HJ72" t="n">
+        <v>105.55</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -40942,6 +41494,21 @@
       <c r="HE73" t="n">
         <v>103</v>
       </c>
+      <c r="HF73" t="n">
+        <v>105</v>
+      </c>
+      <c r="HG73" t="n">
+        <v>100.25</v>
+      </c>
+      <c r="HH73" t="n">
+        <v>100.5</v>
+      </c>
+      <c r="HI73" t="n">
+        <v>100.9</v>
+      </c>
+      <c r="HJ73" t="n">
+        <v>105.5</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -41516,6 +42083,18 @@
       <c r="HE74" t="n">
         <v>103.9</v>
       </c>
+      <c r="HG74" t="n">
+        <v>100.5</v>
+      </c>
+      <c r="HH74" t="n">
+        <v>101.3</v>
+      </c>
+      <c r="HI74" t="n">
+        <v>101</v>
+      </c>
+      <c r="HJ74" t="n">
+        <v>105.3</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">

</xml_diff>